<commit_message>
feat: restructure roles and responsibilities data with detailed activity breakdowns
#VERCEL_SKIP
</commit_message>
<xml_diff>
--- a/public/FPL Staffing.xlsx
+++ b/public/FPL Staffing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pwc-my.sharepoint.com/personal/mayur_murlidhar_kinhekar_pwc_com/Documents/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D49B176-10E3-499B-BB8A-FFE460CAC201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFB0F388-5287-4C2C-8CE4-37F7E929E3D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team Details" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="290">
   <si>
     <t>Name</t>
   </si>
@@ -837,149 +837,6 @@
     <t>Rodolfo</t>
   </si>
   <si>
-    <t>FPL Program – Roles &amp; Responsibilities</t>
-  </si>
-  <si>
-    <t>Responsibilities</t>
-  </si>
-  <si>
-    <t>LEADERSHIP</t>
-  </si>
-  <si>
-    <t>• Own client relationship and overall program health
-• Escalation point for risks, blockers, and strategic decisions
-• Align program goals with client executive stakeholders
-• Review and approve program status, scope changes, and budgets
-• Facilitate steering committee meetings and executive reviews</t>
-  </si>
-  <si>
-    <t>• Define and govern end-to-end technical architecture
-• Establish coding standards, integration patterns, and design principles
-• Review technical designs and approve architectural decisions
-• Resolve cross-pod technical dependencies and conflicts
-• Provide guidance on performance, scalability, and security</t>
-  </si>
-  <si>
-    <t>• Translate business requirements into solution designs
-• Own solution blueprints across value streams
-• Validate technical feasibility of proposed solutions
-• Support Dev Leads with design reviews and technical guidance
-• Bridge gap between business requirements and development teams</t>
-  </si>
-  <si>
-    <t>• Map business processes and identify transformation opportunities
-• Define future-state operating model and capability framework
-• Facilitate requirements workshops with business stakeholders
-• Ensure solutions align with business strategy and process goals
-• Produce business architecture artefacts (process maps, RACI, etc.)</t>
-  </si>
-  <si>
-    <t>• Maintain program plan, milestones, and RAID log
-• Track and report on program status, budget, and resource utilisation
-• Coordinate cross-team dependencies and sprint planning
-• Manage change control, governance artefacts, and meeting cadence
-• Support onboarding, off-boarding, and resource management</t>
-  </si>
-  <si>
-    <t>CROSS-FUNCTIONAL PODS</t>
-  </si>
-  <si>
-    <t>• Own integration architecture across all value streams and releases
-• Define API contracts, data mapping standards, and middleware patterns
-• Review and approve integration designs before development
-• Manage integration dependencies between pods and external systems
-• Coordinate integration testing strategy with QA Leads</t>
-  </si>
-  <si>
-    <t>• Build and maintain APIs, middleware, and integration components
-• Execute integration development per approved design
-• Debug and resolve integration defects and data issues
-• Participate in integration SIT/UAT support activities
-• Document integration flows and technical specifications</t>
-  </si>
-  <si>
-    <t>• Own CI/CD pipeline design, tooling, and governance
-• Manage infrastructure provisioning and environment strategy
-• Define branching strategy, release management, and deployment playbooks
-• Oversee platform stability, monitoring, and incident response
-• Ensure security, compliance, and access controls across environments</t>
-  </si>
-  <si>
-    <t>• Build and maintain CI/CD pipelines and automation scripts
-• Manage environment configuration and infrastructure-as-code
-• Support deployment activities across all releases
-• Monitor system health and respond to alerts and incidents
-• Troubleshoot build, deployment, and environment issues</t>
-  </si>
-  <si>
-    <t>• Own Windsurf AI-assisted development tooling setup and adoption
-• Conduct performance profiling and identify bottlenecks across pods
-• Define and enforce performance benchmarks and SLAs
-• Implement performance fixes and optimisations
-• Share best practices and enablement across development teams</t>
-  </si>
-  <si>
-    <t>DEVELOPMENT PODS</t>
-  </si>
-  <si>
-    <t>• Lead day-to-day delivery of the pod's value stream(s)
-• Own sprint planning, story grooming, and task assignment for the pod
-• Review code, enforce standards, and approve pull requests
-• Identify and escalate technical risks and blockers
-• Coordinate with Onshore/Offshore SA on requirement clarity
-• Track pod velocity and report progress to Engagement Lead</t>
-  </si>
-  <si>
-    <t>Onshore SA
-(Solution Analyst)</t>
-  </si>
-  <si>
-    <t>• Translate functional requirements into detailed user stories and acceptance criteria
-• Serve as primary liaison between business stakeholders and the dev pod
-• Facilitate requirement walkthroughs, demos, and sign-offs
-• Maintain functional specification documents and traceability matrix
-• Support UAT by clarifying requirements and validating test cases
-• Identify functional gaps and raise change requests as needed</t>
-  </si>
-  <si>
-    <t>Offshore SA
-(Solution Analyst)</t>
-  </si>
-  <si>
-    <t>• Support Onshore SA in requirements analysis and documentation
-• Prepare detailed functional designs and process flow diagrams
-• Perform functional review of developed features against requirements
-• Coordinate with offshore dev team on requirement queries
-• Assist in defect triage and requirement clarification during SIT/UAT</t>
-  </si>
-  <si>
-    <t>• Design, build, and unit-test features per user stories and technical design
-• Follow coding standards, branching strategy, and peer review process
-• Participate in sprint ceremonies (planning, standups, retrospectives)
-• Fix defects raised during SIT/UAT within agreed SLAs
-• Document code, APIs, and configuration changes
-• Support deployments and post-deployment validation</t>
-  </si>
-  <si>
-    <t>QA / SIT / UAT</t>
-  </si>
-  <si>
-    <t>• Own the test strategy, test plan, and QA governance for all value streams
-• Allocate QA resources across value streams and manage bandwidth
-• Define entry/exit criteria for SIT and UAT phases
-• Track and report defect metrics, test coverage, and release readiness
-• Escalate critical defects and coordinate with Dev Leads for resolution
-• Facilitate UAT sessions with business stakeholders</t>
-  </si>
-  <si>
-    <t>• Author, review, and execute test cases for assigned value streams
-• Perform functional, regression, and integration testing
-• Log defects with clear steps to reproduce, severity, and evidence
-• Retest fixed defects and confirm closure before release
-• Maintain test artefacts (test cases, execution logs, traceability)
-• Support UAT by guiding business users through test scenarios</t>
-  </si>
-  <si>
     <t>Russell Stein</t>
   </si>
   <si>
@@ -993,6 +850,100 @@
   </si>
   <si>
     <t>Administrative</t>
+  </si>
+  <si>
+    <t>FPL Program – Roles &amp; Responsibilities (Derived from RACI)</t>
+  </si>
+  <si>
+    <t>Responsibilities  (R = Responsible · A = Accountable for these activities)</t>
+  </si>
+  <si>
+    <t>ONSHORE SOLUTION ANALYST</t>
+  </si>
+  <si>
+    <t>• Requirements  |  Gather &amp; own requirements (R); accountable for detailing, sign-off, and intake validation (A)
+• Design  |  Accountable for Functional Design, FPL Solution Review, Decision Review Board, and Design Sign-off (A); lead Solution Workshops (R)
+• Development  |  Drive SME reviews to validate built features against requirements (R)
+• SIT  |  Accountable for Test Planning; lead Defect Triage alongside QA (R)
+• UAT  |  Lead UAT Coordination (R); accountable for Business Validation (A)
+• Post-Dev  |  Capture and log feedback in JIRA (R)
+• Sprint Ceremonies  |  Drive Daily Standup, Sprint Planning, and Sprint Demo (R)
+• Hypercare  |  Lead Incident Triage for production issues (R)</t>
+  </si>
+  <si>
+    <t>OFFSHORE SOLUTION ANALYST</t>
+  </si>
+  <si>
+    <t>• Requirements  |  Responsible for Requirement Detailing, Requirement Sign-off, and Intake Validation (R)
+• Design  |  Own Functional Design documentation and Design Sign-off (R)
+• Development  |  Maintain all documentation on Confluence and tracking tools (R)
+• SIT  |  Own Test Planning documentation; participate in Defect Triage (R)
+• Hypercare  |  Co-lead Incident Triage alongside Onshore SA (R)</t>
+  </si>
+  <si>
+    <t>DEVELOPER</t>
+  </si>
+  <si>
+    <t>• Design  |  Own Technical Approach Documentation (R)
+• Development  |  Build and configure all features (R); execute Unit Testing, PMD Code Scans, and Peer Reviews (R)
+• SIT  |  Perform Smoke Testing post-deployment (R); execute Defect Resolution during test cycles (R)
+• UAT  |  Resolve defects raised by business during UAT (R)</t>
+  </si>
+  <si>
+    <t>DEVELOPMENT LEAD</t>
+  </si>
+  <si>
+    <t>• Requirements  |  Accountable for Intake Validation outcomes (A)
+• Design  |  Own Architecture Review (R/A); responsible for FPL Solution Review, Decision Review Board, and Design Sign-off (R); accountable for Technical Approach, Effort Estimation, and Technical Design (A)
+• Development  |  Accountable for Build &amp; Configuration, Unit Testing, PMD Scans, Peer Review, SME Review, and Documentation (A)
+• SIT  |  Accountable for Smoke Testing and Defect Triage resolution (A)
+• UAT  |  Accountable for Defect Resolution during UAT (A)
+• Cutover &amp; Go-Live  |  Responsible for Cutover Planning and Go-live Coordination (R)
+• Hypercare  |  Accountable for Incident Triage and Bug Fixing resolution (A)</t>
+  </si>
+  <si>
+    <t>QUALITY ASSURANCE</t>
+  </si>
+  <si>
+    <t>• SIT  |  Execute Test Execution across all value streams (R); actively participate in Defect Triage (R); validate Environment Readiness and Integration readiness (C)
+• UAT  |  Responsible for Business Validation testing (R)
+• Post-Dev  |  Capture feedback and defects in JIRA post-release (R)
+• Hypercare  |  Participate in Incident Triage and Bug Fixing validation (C)</t>
+  </si>
+  <si>
+    <t>INTEGRATION POD</t>
+  </si>
+  <si>
+    <t>• Requirements &amp; Design  |  Consulted on all requirements, architecture, and design activities to ensure integration alignment (C)
+• Development  |  Consulted on Technical Design; ensure integration components are factored into build (C)
+• SIT  |  Own Integration Validation end-to-end (R/A); participate in Defect Triage (C)
+• Cutover &amp; Go-Live  |  Consulted on Cutover Planning and Go-live Coordination (C)
+• Hypercare  |  Participate in Incident Triage; support integration-related bug fixes (C)</t>
+  </si>
+  <si>
+    <t>DEVOPS POD</t>
+  </si>
+  <si>
+    <t>• SIT  |  Own Code Promotion to Test and Deployment Validation (R/A); own Environment Readiness (R/A)
+• UAT  |  Support environment stability and readiness for UAT execution
+• Cutover  |  Responsible for Deployment Execution and contribute to Cutover Planning (R/A)
+• Go-Live  |  Responsible for Go-live deployment execution (R)
+• Hypercare  |  Monitor production environment health post go-live (C)</t>
+  </si>
+  <si>
+    <t>PROGRAM MANAGEMENT OFFICE (PMO)</t>
+  </si>
+  <si>
+    <t>• Requirements  |  Own Intake Tracking and status reporting (R/A)
+• SIT  |  Accountable for overall Test Execution governance (A)
+• UAT  |  Accountable for UAT Coordination and Progress Tracking (A/R)
+• Cutover &amp; Go-Live  |  Accountable for Cutover Planning, Readiness Checklist, and Go-live Coordination (A)
+• Post-Dev  |  Accountable for Feedback Capture in JIRA and Continuous Improvement Tracking (A/R)
+• Sprint Ceremonies  |  Accountable for Daily Standup, Sprint Planning, and Sprint Demo cadence (A)
+• Hypercare  |  Own Reporting on production issues and resolution status (R/A)</t>
+  </si>
+  <si>
+    <t>RACI Key:  R = Responsible (does the work)   ·   A = Accountable (owns the outcome)   ·   C = Consulted   ·   I = Informed</t>
   </si>
 </sst>
 </file>
@@ -1035,28 +986,29 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
+      <sz val="13"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF1E293B"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF64748B"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1065,22 +1017,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F2D3D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF1E3A5F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0E7C86"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1A56DB"/>
       </patternFill>
     </fill>
     <fill>
@@ -1091,6 +1028,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1D4ED8"/>
       </patternFill>
     </fill>
   </fills>
@@ -1119,16 +1066,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFBFDBFE"/>
+        <color rgb="FFCBD5E1"/>
       </left>
       <right style="thin">
-        <color rgb="FFBFDBFE"/>
+        <color rgb="FFCBD5E1"/>
       </right>
       <top style="thin">
-        <color rgb="FFBFDBFE"/>
+        <color rgb="FFCBD5E1"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFBFDBFE"/>
+        <color rgb="FFCBD5E1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1138,7 +1085,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1148,32 +1095,29 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="16" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1522,28 +1466,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1554,7 +1498,7 @@
       <c r="B2" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="5" t="s">
         <v>245</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -1578,7 +1522,7 @@
       <c r="B3" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="5" t="s">
         <v>245</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -1833,7 +1777,7 @@
       <c r="G13" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="H13" s="13"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
@@ -2049,7 +1993,7 @@
       <c r="G22" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H22" s="13"/>
+      <c r="H22" s="6"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
@@ -2951,7 +2895,7 @@
       <c r="A61" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="B61" s="14"/>
+      <c r="B61" s="7"/>
       <c r="C61" s="2" t="s">
         <v>10</v>
       </c>
@@ -2973,7 +2917,7 @@
       <c r="A62" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B62" s="14" t="s">
+      <c r="B62" s="7" t="s">
         <v>110</v>
       </c>
       <c r="C62" s="2" t="s">
@@ -3021,7 +2965,7 @@
       <c r="A64" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B64" s="14"/>
+      <c r="B64" s="7"/>
       <c r="C64" s="2" t="s">
         <v>254</v>
       </c>
@@ -3043,7 +2987,7 @@
       <c r="A65" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="B65" s="14"/>
+      <c r="B65" s="7"/>
       <c r="C65" s="2" t="s">
         <v>254</v>
       </c>
@@ -3065,7 +3009,7 @@
       <c r="A66" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="B66" s="14"/>
+      <c r="B66" s="7"/>
       <c r="C66" s="2" t="s">
         <v>254</v>
       </c>
@@ -3135,7 +3079,7 @@
       <c r="A69" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B69" s="14" t="s">
+      <c r="B69" s="7" t="s">
         <v>128</v>
       </c>
       <c r="C69" s="2" t="s">
@@ -3159,7 +3103,7 @@
       <c r="A70" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="B70" s="14"/>
+      <c r="B70" s="7"/>
       <c r="C70" s="2" t="s">
         <v>17</v>
       </c>
@@ -3181,7 +3125,7 @@
       <c r="A71" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B71" s="14" t="s">
+      <c r="B71" s="7" t="s">
         <v>160</v>
       </c>
       <c r="C71" s="2" t="s">
@@ -3205,7 +3149,7 @@
       <c r="A72" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B72" s="14" t="s">
+      <c r="B72" s="7" t="s">
         <v>101</v>
       </c>
       <c r="C72" s="2" t="s">
@@ -3229,7 +3173,7 @@
       <c r="A73" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B73" s="14" t="s">
+      <c r="B73" s="7" t="s">
         <v>126</v>
       </c>
       <c r="C73" s="2" t="s">
@@ -4036,14 +3980,14 @@
       <c r="H106" s="3"/>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A107" s="15" t="s">
+      <c r="A107" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="B107" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="C107" s="16" t="s">
-        <v>294</v>
+      <c r="B107" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="C107" s="8" t="s">
+        <v>270</v>
       </c>
       <c r="D107" s="2" t="s">
         <v>171</v>
@@ -4060,11 +4004,11 @@
       <c r="H107" s="3"/>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A108" s="15" t="s">
-        <v>290</v>
-      </c>
-      <c r="B108" s="12" t="s">
-        <v>291</v>
+      <c r="A108" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>267</v>
       </c>
       <c r="C108" s="3" t="s">
         <v>17</v>
@@ -4078,10 +4022,10 @@
       <c r="F108" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="G108" s="12" t="s">
-        <v>292</v>
-      </c>
-      <c r="H108" s="12"/>
+      <c r="G108" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="H108" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -4127,186 +4071,101 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0FD88A8-2012-4694-A127-A25AEFCD5336}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.81640625" customWidth="1"/>
-    <col min="2" max="2" width="102.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.08984375" customWidth="1"/>
+    <col min="2" max="2" width="88.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="B1" s="6"/>
+    <row r="1" spans="1:2" ht="17" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" s="9"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="B3" s="6"/>
+      <c r="B2" s="11" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="117" x14ac:dyDescent="0.35">
+      <c r="A3" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>274</v>
+      </c>
     </row>
     <row r="4" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>269</v>
+      <c r="A4" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>271</v>
+      <c r="A5" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="117" x14ac:dyDescent="0.35">
+      <c r="A6" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
-        <v>274</v>
-      </c>
-      <c r="B9" s="6"/>
-    </row>
-    <row r="10" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A11" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
-        <v>280</v>
-      </c>
-      <c r="B15" s="6"/>
-    </row>
-    <row r="16" spans="1:2" ht="78" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="B16" s="10" t="s">
+      <c r="A7" s="12" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="78" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
+      <c r="B7" s="13" t="s">
         <v>282</v>
       </c>
-      <c r="B17" s="11" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="78" x14ac:dyDescent="0.35">
+      <c r="A8" s="12" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
+      <c r="B8" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="B18" s="10" t="s">
+    </row>
+    <row r="9" spans="1:2" ht="65" x14ac:dyDescent="0.35">
+      <c r="A9" s="12" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" ht="78" x14ac:dyDescent="0.35">
-      <c r="A19" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="B19" s="11" t="s">
+      <c r="B9" s="13" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="8" t="s">
+    <row r="10" spans="1:2" ht="91" x14ac:dyDescent="0.35">
+      <c r="A10" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="B20" s="6"/>
-    </row>
-    <row r="21" spans="1:2" ht="78" x14ac:dyDescent="0.35">
-      <c r="A21" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="B21" s="11" t="s">
+      <c r="B10" s="14" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="78" x14ac:dyDescent="0.35">
-      <c r="A22" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B22" s="10" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="15" t="s">
         <v>289</v>
       </c>
+      <c r="B12" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="2">
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update FPL Staffing spreadsheet
Updated staffing details in Excel file

#VERCEL_SKIP
</commit_message>
<xml_diff>
--- a/public/FPL Staffing.xlsx
+++ b/public/FPL Staffing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pwc-my.sharepoint.com/personal/mayur_murlidhar_kinhekar_pwc_com/Documents/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFB0F388-5287-4C2C-8CE4-37F7E929E3D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D2C301C-9EFE-4E78-AF8A-4438500D2579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1211" uniqueCount="343">
   <si>
     <t>Name</t>
   </si>
@@ -852,105 +852,227 @@
     <t>Administrative</t>
   </si>
   <si>
-    <t>FPL Program – Roles &amp; Responsibilities (Derived from RACI)</t>
-  </si>
-  <si>
-    <t>Responsibilities  (R = Responsible · A = Accountable for these activities)</t>
-  </si>
-  <si>
-    <t>ONSHORE SOLUTION ANALYST</t>
-  </si>
-  <si>
-    <t>• Requirements  |  Gather &amp; own requirements (R); accountable for detailing, sign-off, and intake validation (A)
-• Design  |  Accountable for Functional Design, FPL Solution Review, Decision Review Board, and Design Sign-off (A); lead Solution Workshops (R)
-• Development  |  Drive SME reviews to validate built features against requirements (R)
-• SIT  |  Accountable for Test Planning; lead Defect Triage alongside QA (R)
-• UAT  |  Lead UAT Coordination (R); accountable for Business Validation (A)
-• Post-Dev  |  Capture and log feedback in JIRA (R)
-• Sprint Ceremonies  |  Drive Daily Standup, Sprint Planning, and Sprint Demo (R)
-• Hypercare  |  Lead Incident Triage for production issues (R)</t>
-  </si>
-  <si>
-    <t>OFFSHORE SOLUTION ANALYST</t>
-  </si>
-  <si>
-    <t>• Requirements  |  Responsible for Requirement Detailing, Requirement Sign-off, and Intake Validation (R)
-• Design  |  Own Functional Design documentation and Design Sign-off (R)
-• Development  |  Maintain all documentation on Confluence and tracking tools (R)
-• SIT  |  Own Test Planning documentation; participate in Defect Triage (R)
-• Hypercare  |  Co-lead Incident Triage alongside Onshore SA (R)</t>
-  </si>
-  <si>
-    <t>DEVELOPER</t>
-  </si>
-  <si>
-    <t>• Design  |  Own Technical Approach Documentation (R)
-• Development  |  Build and configure all features (R); execute Unit Testing, PMD Code Scans, and Peer Reviews (R)
-• SIT  |  Perform Smoke Testing post-deployment (R); execute Defect Resolution during test cycles (R)
-• UAT  |  Resolve defects raised by business during UAT (R)</t>
-  </si>
-  <si>
-    <t>DEVELOPMENT LEAD</t>
-  </si>
-  <si>
-    <t>• Requirements  |  Accountable for Intake Validation outcomes (A)
-• Design  |  Own Architecture Review (R/A); responsible for FPL Solution Review, Decision Review Board, and Design Sign-off (R); accountable for Technical Approach, Effort Estimation, and Technical Design (A)
-• Development  |  Accountable for Build &amp; Configuration, Unit Testing, PMD Scans, Peer Review, SME Review, and Documentation (A)
-• SIT  |  Accountable for Smoke Testing and Defect Triage resolution (A)
-• UAT  |  Accountable for Defect Resolution during UAT (A)
-• Cutover &amp; Go-Live  |  Responsible for Cutover Planning and Go-live Coordination (R)
-• Hypercare  |  Accountable for Incident Triage and Bug Fixing resolution (A)</t>
-  </si>
-  <si>
-    <t>QUALITY ASSURANCE</t>
-  </si>
-  <si>
-    <t>• SIT  |  Execute Test Execution across all value streams (R); actively participate in Defect Triage (R); validate Environment Readiness and Integration readiness (C)
-• UAT  |  Responsible for Business Validation testing (R)
-• Post-Dev  |  Capture feedback and defects in JIRA post-release (R)
-• Hypercare  |  Participate in Incident Triage and Bug Fixing validation (C)</t>
-  </si>
-  <si>
-    <t>INTEGRATION POD</t>
-  </si>
-  <si>
-    <t>• Requirements &amp; Design  |  Consulted on all requirements, architecture, and design activities to ensure integration alignment (C)
-• Development  |  Consulted on Technical Design; ensure integration components are factored into build (C)
-• SIT  |  Own Integration Validation end-to-end (R/A); participate in Defect Triage (C)
-• Cutover &amp; Go-Live  |  Consulted on Cutover Planning and Go-live Coordination (C)
-• Hypercare  |  Participate in Incident Triage; support integration-related bug fixes (C)</t>
-  </si>
-  <si>
-    <t>DEVOPS POD</t>
-  </si>
-  <si>
-    <t>• SIT  |  Own Code Promotion to Test and Deployment Validation (R/A); own Environment Readiness (R/A)
-• UAT  |  Support environment stability and readiness for UAT execution
-• Cutover  |  Responsible for Deployment Execution and contribute to Cutover Planning (R/A)
-• Go-Live  |  Responsible for Go-live deployment execution (R)
-• Hypercare  |  Monitor production environment health post go-live (C)</t>
-  </si>
-  <si>
-    <t>PROGRAM MANAGEMENT OFFICE (PMO)</t>
-  </si>
-  <si>
-    <t>• Requirements  |  Own Intake Tracking and status reporting (R/A)
-• SIT  |  Accountable for overall Test Execution governance (A)
-• UAT  |  Accountable for UAT Coordination and Progress Tracking (A/R)
-• Cutover &amp; Go-Live  |  Accountable for Cutover Planning, Readiness Checklist, and Go-live Coordination (A)
-• Post-Dev  |  Accountable for Feedback Capture in JIRA and Continuous Improvement Tracking (A/R)
-• Sprint Ceremonies  |  Accountable for Daily Standup, Sprint Planning, and Sprint Demo cadence (A)
-• Hypercare  |  Own Reporting on production issues and resolution status (R/A)</t>
-  </si>
-  <si>
-    <t>RACI Key:  R = Responsible (does the work)   ·   A = Accountable (owns the outcome)   ·   C = Consulted   ·   I = Informed</t>
+    <t>Lifecycle Phase</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>Onshore Solution Analyst</t>
+  </si>
+  <si>
+    <t>Offshore Solution Analyst</t>
+  </si>
+  <si>
+    <t>Developer</t>
+  </si>
+  <si>
+    <t>Development Lead</t>
+  </si>
+  <si>
+    <t>Quality Assurance</t>
+  </si>
+  <si>
+    <t>Integration POD</t>
+  </si>
+  <si>
+    <t>DevOps POD</t>
+  </si>
+  <si>
+    <t>Program Management Office</t>
+  </si>
+  <si>
+    <t>Requirements</t>
+  </si>
+  <si>
+    <t>Requirement Gathering</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Requirement Detailing</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Requirement Sign-off</t>
+  </si>
+  <si>
+    <t>Intake Validation</t>
+  </si>
+  <si>
+    <t>Intake Tracking</t>
+  </si>
+  <si>
+    <t>R/A</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Technical Approach Documentation</t>
+  </si>
+  <si>
+    <t>Architecture Review</t>
+  </si>
+  <si>
+    <t>FPL Solution Review</t>
+  </si>
+  <si>
+    <t>Decision Review Board</t>
+  </si>
+  <si>
+    <t>Functional Design</t>
+  </si>
+  <si>
+    <t>Technical Design</t>
+  </si>
+  <si>
+    <t>Solution Workshops</t>
+  </si>
+  <si>
+    <t>Effort Estimation</t>
+  </si>
+  <si>
+    <t>Design Sign-off</t>
+  </si>
+  <si>
+    <t>Development</t>
+  </si>
+  <si>
+    <t>Build &amp; Configuration</t>
+  </si>
+  <si>
+    <t>Unit Testing</t>
+  </si>
+  <si>
+    <t>PMD Code Scan</t>
+  </si>
+  <si>
+    <t>Peer Review</t>
+  </si>
+  <si>
+    <t>UI/UX Review</t>
+  </si>
+  <si>
+    <t>SME Review</t>
+  </si>
+  <si>
+    <t>Documentation (Confluence &amp; Tracker)</t>
+  </si>
+  <si>
+    <t>SIT</t>
+  </si>
+  <si>
+    <t>Code Promotion to Test</t>
+  </si>
+  <si>
+    <t>Smoke Testing</t>
+  </si>
+  <si>
+    <t>Deployment Validation</t>
+  </si>
+  <si>
+    <t>Test Planning</t>
+  </si>
+  <si>
+    <t>Test Execution</t>
+  </si>
+  <si>
+    <t>Defect Triage</t>
+  </si>
+  <si>
+    <t>Integration Validation</t>
+  </si>
+  <si>
+    <t>Environment Readiness</t>
+  </si>
+  <si>
+    <t>UAT</t>
+  </si>
+  <si>
+    <t>UAT Coordination</t>
+  </si>
+  <si>
+    <t>Business Validation</t>
+  </si>
+  <si>
+    <t>Defect Resolution</t>
+  </si>
+  <si>
+    <t>Progress Tracking</t>
+  </si>
+  <si>
+    <t>Cutover</t>
+  </si>
+  <si>
+    <t>Cutover Planning</t>
+  </si>
+  <si>
+    <t>Deployment Execution</t>
+  </si>
+  <si>
+    <t>Readiness Checklist</t>
+  </si>
+  <si>
+    <t>Go Live</t>
+  </si>
+  <si>
+    <t>Go-live Coordination</t>
+  </si>
+  <si>
+    <t>Post-Dev</t>
+  </si>
+  <si>
+    <t>Feedback Capture (JIRA)</t>
+  </si>
+  <si>
+    <t>Continuous Improvement Tracking</t>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>Daily Standup</t>
+  </si>
+  <si>
+    <t>Sprint Planning</t>
+  </si>
+  <si>
+    <t>Sprint Demo</t>
+  </si>
+  <si>
+    <t>Hypercare</t>
+  </si>
+  <si>
+    <t>Incident Triage</t>
+  </si>
+  <si>
+    <t>Bug Fixing</t>
+  </si>
+  <si>
+    <t>Production Monitoring</t>
+  </si>
+  <si>
+    <t>Reporting</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -986,29 +1108,17 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF1E293B"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="9"/>
-      <color rgb="FF64748B"/>
-      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1017,31 +1127,60 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1E3A5F"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEFF6FF"/>
+        <fgColor rgb="FFCFE2F3"/>
+        <bgColor rgb="FFCFE2F3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0F172A"/>
+        <fgColor rgb="FFFCE5CD"/>
+        <bgColor rgb="FFFCE5CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1D4ED8"/>
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0E0E3"/>
+        <bgColor rgb="FFD0E0E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor rgb="FFF4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D2E9"/>
+        <bgColor rgb="FFD9D2E9"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1064,28 +1203,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1099,25 +1223,18 @@
     <xf numFmtId="16" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4071,102 +4188,1526 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0FD88A8-2012-4694-A127-A25AEFCD5336}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.08984375" customWidth="1"/>
-    <col min="2" max="2" width="88.1796875" customWidth="1"/>
+    <col min="1" max="1" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="17" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="9"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="11" t="s">
+      <c r="B1" s="9" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="117" x14ac:dyDescent="0.35">
-      <c r="A3" s="12" t="s">
+      <c r="C1" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="D1" s="9" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A4" s="12" t="s">
+      <c r="E1" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="F1" s="9" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
+      <c r="G1" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="H1" s="9" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="117" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
+      <c r="I1" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="J1" s="9" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A7" s="12" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B2" s="10" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="78" x14ac:dyDescent="0.35">
-      <c r="A8" s="12" t="s">
+      <c r="C2" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="B8" s="14" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="65" x14ac:dyDescent="0.35">
-      <c r="A9" s="12" t="s">
-        <v>285</v>
-      </c>
-      <c r="B9" s="13" t="s">
+      <c r="D2" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="I2" s="10" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="91" x14ac:dyDescent="0.35">
-      <c r="A10" s="12" t="s">
+      <c r="J2" s="10" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="C3" s="10" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="15" t="s">
+      <c r="D3" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="B12" s="9"/>
+      <c r="C4" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>292</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>298</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="J11" s="11" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>304</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="I16" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="J16" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>305</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="J17" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="J19" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="I20" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="I21" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="J21" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="I22" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="I23" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="J23" s="13" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="G24" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="I24" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="J24" s="13" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="G25" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="I25" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="I26" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>316</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="G27" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="H27" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="I27" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="J27" s="13" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>317</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="G28" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="H28" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="I28" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="J28" s="13" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="G29" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="H29" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="I29" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="J29" s="13" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>319</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="G30" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="H30" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="I30" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>321</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="G31" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="H31" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="I31" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="J31" s="14" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>322</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="F32" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="G32" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="J32" s="14" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>323</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="F33" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="G33" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="H33" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="I33" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="J33" s="14" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A34" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>324</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="F34" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="G34" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="I34" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="J34" s="14" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A35" s="15" t="s">
+        <v>325</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>283</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>283</v>
+      </c>
+      <c r="J35" s="15" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A36" s="15" t="s">
+        <v>325</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>327</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="F36" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="H36" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="I36" s="15" t="s">
+        <v>292</v>
+      </c>
+      <c r="J36" s="15" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A37" s="15" t="s">
+        <v>325</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>328</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="F37" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="G37" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="I37" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="J37" s="15" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A38" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="I38" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="J38" s="10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A39" s="16" t="s">
+        <v>331</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>332</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>283</v>
+      </c>
+      <c r="D39" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="E39" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="F39" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="G39" s="16" t="s">
+        <v>283</v>
+      </c>
+      <c r="H39" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="I39" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="J39" s="16" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A40" s="16" t="s">
+        <v>331</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>285</v>
+      </c>
+      <c r="D40" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="E40" s="16" t="s">
+        <v>285</v>
+      </c>
+      <c r="F40" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="G40" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="H40" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="I40" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="J40" s="16" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A41" s="17" t="s">
+        <v>334</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>335</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="D41" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="E41" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="F41" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="G41" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="H41" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="I41" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="J41" s="17" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A42" s="17" t="s">
+        <v>334</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>336</v>
+      </c>
+      <c r="C42" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="D42" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="E42" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="F42" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="G42" s="17" t="s">
+        <v>285</v>
+      </c>
+      <c r="H42" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="I42" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="J42" s="17" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A43" s="17" t="s">
+        <v>334</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>337</v>
+      </c>
+      <c r="C43" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="D43" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="E43" s="17" t="s">
+        <v>285</v>
+      </c>
+      <c r="F43" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="G43" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="H43" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="I43" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="J43" s="17" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A44" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>339</v>
+      </c>
+      <c r="C44" s="18" t="s">
+        <v>283</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>283</v>
+      </c>
+      <c r="E44" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="F44" s="18" t="s">
+        <v>288</v>
+      </c>
+      <c r="G44" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="H44" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="I44" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="J44" s="18" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A45" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="C45" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="E45" s="18" t="s">
+        <v>283</v>
+      </c>
+      <c r="F45" s="18" t="s">
+        <v>288</v>
+      </c>
+      <c r="G45" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="H45" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="I45" s="18" t="s">
+        <v>286</v>
+      </c>
+      <c r="J45" s="18" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A46" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="C46" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="D46" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="E46" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="F46" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="G46" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="H46" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="I46" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="J46" s="18" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A47" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>342</v>
+      </c>
+      <c r="C47" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="D47" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="E47" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="F47" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="G47" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="H47" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="I47" s="18" t="s">
+        <v>286</v>
+      </c>
+      <c r="J47" s="18" t="s">
+        <v>292</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A12:B12"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update FPL Staffing.xlsx file with new data
Updated staffing details for FPL team

#VERCEL_SKIP
</commit_message>
<xml_diff>
--- a/public/FPL Staffing.xlsx
+++ b/public/FPL Staffing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pwc-my.sharepoint.com/personal/mayur_murlidhar_kinhekar_pwc_com/Documents/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D2C301C-9EFE-4E78-AF8A-4438500D2579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{661011C8-39E0-4996-8ACC-79CD5315E4B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team Details" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1211" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="353">
   <si>
     <t>Name</t>
   </si>
@@ -1066,6 +1066,36 @@
   </si>
   <si>
     <t>Reporting</t>
+  </si>
+  <si>
+    <t>Ziyad Auti</t>
+  </si>
+  <si>
+    <t>Kishor S</t>
+  </si>
+  <si>
+    <t>Krithika Harishchandra Shettigar</t>
+  </si>
+  <si>
+    <t>Potumanchi Sree Yashana</t>
+  </si>
+  <si>
+    <t>Adithya Sankar S</t>
+  </si>
+  <si>
+    <t>ziyad.auti@pwc.com</t>
+  </si>
+  <si>
+    <t>kishor.selvakumar@pwc.com</t>
+  </si>
+  <si>
+    <t>krithika.h.shettigar@pwc.com</t>
+  </si>
+  <si>
+    <t>potumanchi.sree.yashana@pwc.com</t>
+  </si>
+  <si>
+    <t>adithya.sankar.s@pwc.com</t>
   </si>
 </sst>
 </file>
@@ -1571,10 +1601,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FD4BB79-FFCA-43BE-A86E-E3939215755C}">
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.1796875" customWidth="1"/>
+    <col min="1" max="1" width="34.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="43.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
@@ -4143,6 +4173,116 @@
         <v>268</v>
       </c>
       <c r="H108" s="5"/>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A109" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="C109" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G109" s="3"/>
+      <c r="H109" s="3"/>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A110" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="C110" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G110" s="3"/>
+      <c r="H110" s="3"/>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A111" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="C111" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G111" s="3"/>
+      <c r="H111" s="3"/>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A112" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="C112" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D112" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G112" s="3"/>
+      <c r="H112" s="3"/>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A113" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C113" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D113" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G113" s="3"/>
+      <c r="H113" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
chore: update FPL Staffing.xlsx file
Updated staffing file with latest data.

#VERCEL_SKIP
</commit_message>
<xml_diff>
--- a/public/FPL Staffing.xlsx
+++ b/public/FPL Staffing.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I159"/>
+  <dimension ref="A1:I153"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1214,13 +1214,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Ambati Venkata Sai Harika</v>
+        <v>Ankit Mishra</v>
       </c>
       <c r="B29" t="str">
-        <v>venkata.sai.harika.ambati@pwc.com</v>
+        <v>ankit.b.mishra@pwc.com</v>
       </c>
       <c r="C29" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D29" t="str">
         <v>Dev</v>
@@ -1232,7 +1232,7 @@
         <v>IR4</v>
       </c>
       <c r="G29" t="str">
-        <v>Energy Management</v>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -1243,13 +1243,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Ankit Mishra</v>
+        <v>Ankit Verma</v>
       </c>
       <c r="B30" t="str">
-        <v>ankit.b.mishra@pwc.com</v>
+        <v/>
       </c>
       <c r="C30" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D30" t="str">
         <v>Dev</v>
@@ -1261,10 +1261,10 @@
         <v>IR4</v>
       </c>
       <c r="G30" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v/>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I30" t="str">
         <v>No</v>
@@ -1272,13 +1272,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Ankit Prasad Verma</v>
+        <v>Chaitra Hanchinal</v>
       </c>
       <c r="B31" t="str">
-        <v>ankit.prasad.verma@pwc.com</v>
+        <v/>
       </c>
       <c r="C31" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D31" t="str">
         <v>Dev</v>
@@ -1290,10 +1290,10 @@
         <v>IR4</v>
       </c>
       <c r="G31" t="str">
-        <v>Case Management</v>
+        <v/>
       </c>
       <c r="H31" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I31" t="str">
         <v>No</v>
@@ -1301,13 +1301,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Ankit Verma</v>
+        <v>Cheruku Pranay Reddy</v>
       </c>
       <c r="B32" t="str">
-        <v/>
+        <v>cheruku.pranay.reddy@pwc.com</v>
       </c>
       <c r="C32" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D32" t="str">
         <v>Dev</v>
@@ -1319,10 +1319,10 @@
         <v>IR4</v>
       </c>
       <c r="G32" t="str">
-        <v/>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H32" t="str">
-        <v>Case Management POD</v>
+        <v/>
       </c>
       <c r="I32" t="str">
         <v>No</v>
@@ -1330,13 +1330,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Chaitra Hanchinal</v>
+        <v>Jaya Lakshmi Papolu</v>
       </c>
       <c r="B33" t="str">
-        <v>chaitra.s.hanchinal@pwc.com</v>
+        <v/>
       </c>
       <c r="C33" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D33" t="str">
         <v>Dev</v>
@@ -1348,7 +1348,7 @@
         <v>IR4</v>
       </c>
       <c r="G33" t="str">
-        <v>Field Management</v>
+        <v/>
       </c>
       <c r="H33" t="str">
         <v>Field Management POD</v>
@@ -1359,10 +1359,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Cheruku Pranay Reddy</v>
+        <v>Jayoti Chatterji</v>
       </c>
       <c r="B34" t="str">
-        <v>cheruku.pranay.reddy@pwc.com</v>
+        <v>jayoti.chatterji@pwc.com</v>
       </c>
       <c r="C34" t="str">
         <v>Senior Associate</v>
@@ -1371,16 +1371,16 @@
         <v>Dev</v>
       </c>
       <c r="E34" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="F34" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="G34" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Outage</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I34" t="str">
         <v>No</v>
@@ -1388,13 +1388,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Jaya Lakshmi Papolu</v>
+        <v>John Jyothula</v>
       </c>
       <c r="B35" t="str">
-        <v>jaya.lakshmi.papolu@pwc.com</v>
+        <v/>
       </c>
       <c r="C35" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D35" t="str">
         <v>Dev</v>
@@ -1406,10 +1406,10 @@
         <v>IR4</v>
       </c>
       <c r="G35" t="str">
-        <v>Field Management</v>
+        <v/>
       </c>
       <c r="H35" t="str">
-        <v>Field Management POD</v>
+        <v>Case Management POD</v>
       </c>
       <c r="I35" t="str">
         <v>No</v>
@@ -1417,28 +1417,28 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Jayoti Chatterji</v>
+        <v>Kankshitha Yalamuru</v>
       </c>
       <c r="B36" t="str">
-        <v>jayoti.chatterji@pwc.com</v>
+        <v/>
       </c>
       <c r="C36" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D36" t="str">
         <v>Dev</v>
       </c>
       <c r="E36" t="str">
-        <v>IR3.X</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F36" t="str">
-        <v>IR3.X</v>
+        <v>All</v>
       </c>
       <c r="G36" t="str">
-        <v>Outage</v>
+        <v/>
       </c>
       <c r="H36" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v/>
       </c>
       <c r="I36" t="str">
         <v>No</v>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>John Jyothula</v>
+        <v>Kavita Jha</v>
       </c>
       <c r="B37" t="str">
         <v/>
@@ -1467,7 +1467,7 @@
         <v/>
       </c>
       <c r="H37" t="str">
-        <v>Case Management POD</v>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I37" t="str">
         <v>No</v>
@@ -1475,10 +1475,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Jyothula John Paramjyothi</v>
+        <v>Madhumita Kodidela</v>
       </c>
       <c r="B38" t="str">
-        <v>john.paramjyothi.jyothula@pwc.com</v>
+        <v>madhumitha.kodidela@pwc.com</v>
       </c>
       <c r="C38" t="str">
         <v>Senior Associate</v>
@@ -1487,16 +1487,16 @@
         <v>Dev</v>
       </c>
       <c r="E38" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F38" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G38" t="str">
-        <v>Case Management</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H38" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I38" t="str">
         <v>No</v>
@@ -1504,25 +1504,25 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Kankshitha Yalamuru</v>
+        <v>Manu Tyagi</v>
       </c>
       <c r="B39" t="str">
-        <v>yalamuru.sai.kankshitha@pwc.com</v>
+        <v/>
       </c>
       <c r="C39" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D39" t="str">
         <v>Dev</v>
       </c>
       <c r="E39" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F39" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G39" t="str">
-        <v>Billing &amp; Usage</v>
+        <v/>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -1533,10 +1533,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Kavita Jha</v>
+        <v>Mounika Depuri</v>
       </c>
       <c r="B40" t="str">
-        <v>kavita.jha@pwc.com</v>
+        <v>mounika.depuri@pwc.com</v>
       </c>
       <c r="C40" t="str">
         <v>Senior Associate</v>
@@ -1545,16 +1545,16 @@
         <v>Dev</v>
       </c>
       <c r="E40" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F40" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G40" t="str">
-        <v>Outage</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H40" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v/>
       </c>
       <c r="I40" t="str">
         <v>No</v>
@@ -1562,28 +1562,28 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Madhumita Kodidela</v>
+        <v>Mrithika Kumaresan</v>
       </c>
       <c r="B41" t="str">
-        <v>madhumitha.kodidela@pwc.com</v>
+        <v/>
       </c>
       <c r="C41" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D41" t="str">
         <v>Dev</v>
       </c>
       <c r="E41" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F41" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G41" t="str">
-        <v>Interactions/Search</v>
+        <v/>
       </c>
       <c r="H41" t="str">
-        <v>Dev POD 2/Sneha G</v>
+        <v>Field Management POD</v>
       </c>
       <c r="I41" t="str">
         <v>No</v>
@@ -1591,10 +1591,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Manu Tyagi</v>
+        <v>Mylavarapu V N R Saketh</v>
       </c>
       <c r="B42" t="str">
-        <v>manu.tyagi@pwc.com</v>
+        <v>mylavarapu.v.n.r.saketh@pwc.com</v>
       </c>
       <c r="C42" t="str">
         <v>Senior Associate</v>
@@ -1609,10 +1609,10 @@
         <v>IR4</v>
       </c>
       <c r="G42" t="str">
-        <v>Interactions/Search</v>
+        <v>Energy Management</v>
       </c>
       <c r="H42" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I42" t="str">
         <v>No</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Mounika Depuri</v>
+        <v>Naman Hiran</v>
       </c>
       <c r="B43" t="str">
-        <v>mounika.depuri@pwc.com</v>
+        <v>naman.hiran@pwc.com</v>
       </c>
       <c r="C43" t="str">
         <v>Senior Associate</v>
@@ -1632,16 +1632,16 @@
         <v>Dev</v>
       </c>
       <c r="E43" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F43" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G43" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Energy Management</v>
       </c>
       <c r="H43" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I43" t="str">
         <v>No</v>
@@ -1649,28 +1649,28 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Mrithika Kumaresan</v>
+        <v>Nishi Jain</v>
       </c>
       <c r="B44" t="str">
-        <v>mrithika.kumaresan@pwc.com</v>
+        <v/>
       </c>
       <c r="C44" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D44" t="str">
         <v>Dev</v>
       </c>
       <c r="E44" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F44" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G44" t="str">
-        <v>Field Management</v>
+        <v/>
       </c>
       <c r="H44" t="str">
-        <v>Field Management POD</v>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I44" t="str">
         <v>No</v>
@@ -1678,10 +1678,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Mylavarapu V N R Saketh</v>
+        <v>Nishi Narendra Jain</v>
       </c>
       <c r="B45" t="str">
-        <v>mylavarapu.v.n.r.saketh@pwc.com</v>
+        <v>jain.u.nishi@pwc.com</v>
       </c>
       <c r="C45" t="str">
         <v>Senior Associate</v>
@@ -1690,16 +1690,16 @@
         <v>Dev</v>
       </c>
       <c r="E45" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F45" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G45" t="str">
-        <v>Energy Management</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H45" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I45" t="str">
         <v>No</v>
@@ -1707,13 +1707,13 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Naman Hiran</v>
+        <v>Nivetha Sudharsanam</v>
       </c>
       <c r="B46" t="str">
-        <v xml:space="preserve">naman.h.hiran@pwc.com </v>
+        <v/>
       </c>
       <c r="C46" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D46" t="str">
         <v>Dev</v>
@@ -1725,10 +1725,10 @@
         <v>IR4</v>
       </c>
       <c r="G46" t="str">
-        <v>Energy Management</v>
+        <v/>
       </c>
       <c r="H46" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I46" t="str">
         <v>No</v>
@@ -1736,13 +1736,13 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Nishi Jain</v>
+        <v>Piyush Singh</v>
       </c>
       <c r="B47" t="str">
-        <v/>
+        <v>piyush.ss.singh@pwc.com</v>
       </c>
       <c r="C47" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D47" t="str">
         <v>Dev</v>
@@ -1754,10 +1754,10 @@
         <v>IR3.2</v>
       </c>
       <c r="G47" t="str">
-        <v/>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H47" t="str">
-        <v>Dev POD 6/Aditya</v>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I47" t="str">
         <v>No</v>
@@ -1765,28 +1765,28 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Nishi Narendra Jain</v>
+        <v>Pradeep Lambu</v>
       </c>
       <c r="B48" t="str">
-        <v>jain.u.nishi@pwc.com</v>
+        <v/>
       </c>
       <c r="C48" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D48" t="str">
         <v>Dev</v>
       </c>
       <c r="E48" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F48" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G48" t="str">
-        <v>Account Maintenance</v>
+        <v/>
       </c>
       <c r="H48" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I48" t="str">
         <v>No</v>
@@ -1794,28 +1794,28 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Nivetha Sudharsanam</v>
+        <v>Pranay Reddy</v>
       </c>
       <c r="B49" t="str">
-        <v>nivetha.sudharsanam@pwc.com</v>
+        <v/>
       </c>
       <c r="C49" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D49" t="str">
         <v>Dev</v>
       </c>
       <c r="E49" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F49" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G49" t="str">
-        <v>Multi Move In/Transfer/Amend</v>
+        <v/>
       </c>
       <c r="H49" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v/>
       </c>
       <c r="I49" t="str">
         <v>No</v>
@@ -1823,28 +1823,28 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Piyush Singh</v>
+        <v>Prasad P</v>
       </c>
       <c r="B50" t="str">
-        <v>piyush.ss.singh@pwc.com</v>
+        <v/>
       </c>
       <c r="C50" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D50" t="str">
         <v>Dev</v>
       </c>
       <c r="E50" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F50" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G50" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v/>
       </c>
       <c r="H50" t="str">
-        <v>Dev POD 4/Suraj</v>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I50" t="str">
         <v>No</v>
@@ -1852,28 +1852,28 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Pradeep L</v>
+        <v>Pratik Kurdukar</v>
       </c>
       <c r="B51" t="str">
-        <v>pradeep.l@pwc.com</v>
+        <v>pratik.k.kurdukar@pwc.com</v>
       </c>
       <c r="C51" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D51" t="str">
         <v>Dev</v>
       </c>
       <c r="E51" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F51" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G51" t="str">
-        <v>Multi Move In/Transfer/Amend</v>
+        <v>Case Management</v>
       </c>
       <c r="H51" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I51" t="str">
         <v>No</v>
@@ -1881,7 +1881,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Pradeep Lambu</v>
+        <v>Rida Maryam Mohammad</v>
       </c>
       <c r="B52" t="str">
         <v/>
@@ -1902,7 +1902,7 @@
         <v/>
       </c>
       <c r="H52" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I52" t="str">
         <v>No</v>
@@ -1910,25 +1910,25 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Pranay Reddy</v>
+        <v>Rubasri S</v>
       </c>
       <c r="B53" t="str">
-        <v/>
+        <v>rubasri.x.s@pwc.com</v>
       </c>
       <c r="C53" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D53" t="str">
         <v>Dev</v>
       </c>
       <c r="E53" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F53" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G53" t="str">
-        <v/>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -1939,28 +1939,28 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Prasad P</v>
+        <v>Sahil Thadani</v>
       </c>
       <c r="B54" t="str">
-        <v>prasad.p@pwc.com</v>
+        <v/>
       </c>
       <c r="C54" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D54" t="str">
         <v>Dev</v>
       </c>
       <c r="E54" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F54" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G54" t="str">
-        <v>Multi Move In/Transfer/Amend</v>
+        <v/>
       </c>
       <c r="H54" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v/>
       </c>
       <c r="I54" t="str">
         <v>No</v>
@@ -1968,28 +1968,28 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Pratik Kurdukar</v>
+        <v>Sahithi Chebrolu</v>
       </c>
       <c r="B55" t="str">
-        <v>pratik.k.kurdukar@pwc.com</v>
+        <v/>
       </c>
       <c r="C55" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D55" t="str">
         <v>Dev</v>
       </c>
       <c r="E55" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F55" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G55" t="str">
-        <v>Case Management</v>
+        <v/>
       </c>
       <c r="H55" t="str">
-        <v>Case Management POD</v>
+        <v/>
       </c>
       <c r="I55" t="str">
         <v>No</v>
@@ -1997,28 +1997,28 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Rida Maryam Mohammad</v>
+        <v>Sandesh Saravanan</v>
       </c>
       <c r="B56" t="str">
-        <v>rida.maryam.mohammad@pwc.com</v>
+        <v>sandesh.saravanan@pwc.com</v>
       </c>
       <c r="C56" t="str">
-        <v>Senior Associate</v>
+        <v>Intern</v>
       </c>
       <c r="D56" t="str">
         <v>Dev</v>
       </c>
       <c r="E56" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F56" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G56" t="str">
-        <v>Outage</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H56" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v>IR3.2 Hypercare Support</v>
       </c>
       <c r="I56" t="str">
         <v>No</v>
@@ -2026,13 +2026,13 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Rubasri S</v>
+        <v>Sanniboina Murali Krishna</v>
       </c>
       <c r="B57" t="str">
-        <v>rubasri.x.s@pwc.com</v>
+        <v/>
       </c>
       <c r="C57" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D57" t="str">
         <v>Dev</v>
@@ -2044,10 +2044,10 @@
         <v>IR4</v>
       </c>
       <c r="G57" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v/>
       </c>
       <c r="H57" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I57" t="str">
         <v>No</v>
@@ -2055,28 +2055,28 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Sahil Thadani</v>
+        <v>Shikhar Sanjeev</v>
       </c>
       <c r="B58" t="str">
-        <v>sahil.kumar.thadani@pwc.com</v>
+        <v>shikhar.sanjeev@pwc.com</v>
       </c>
       <c r="C58" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D58" t="str">
         <v>Dev</v>
       </c>
       <c r="E58" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F58" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G58" t="str">
-        <v>Billing &amp; Usage</v>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H58" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I58" t="str">
         <v>No</v>
@@ -2084,28 +2084,28 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Sandesh Saravanan</v>
+        <v>Shivam Shete</v>
       </c>
       <c r="B59" t="str">
-        <v>sandesh.saravanan@pwc.com</v>
+        <v/>
       </c>
       <c r="C59" t="str">
-        <v>Intern</v>
+        <v/>
       </c>
       <c r="D59" t="str">
         <v>Dev</v>
       </c>
       <c r="E59" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F59" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G59" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v/>
       </c>
       <c r="H59" t="str">
-        <v>IR3.2 Hypercare Support</v>
+        <v/>
       </c>
       <c r="I59" t="str">
         <v>No</v>
@@ -2113,10 +2113,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Sanniboina Murali Krishna</v>
+        <v>Shivam Surendra Shete</v>
       </c>
       <c r="B60" t="str">
-        <v>sanniboina.murali.krishna@pwc.com</v>
+        <v>shivam.surendra.shete@pwc.com</v>
       </c>
       <c r="C60" t="str">
         <v>Senior Associate</v>
@@ -2131,10 +2131,10 @@
         <v>IR4</v>
       </c>
       <c r="G60" t="str">
-        <v>Outage</v>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H60" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v/>
       </c>
       <c r="I60" t="str">
         <v>No</v>
@@ -2142,28 +2142,28 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Shikhar Sanjeev</v>
+        <v>Shravya Nanjundaswamy</v>
       </c>
       <c r="B61" t="str">
-        <v>shikhar.sanjeev@pwc.com</v>
+        <v/>
       </c>
       <c r="C61" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D61" t="str">
         <v>Dev</v>
       </c>
       <c r="E61" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F61" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G61" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v/>
       </c>
       <c r="H61" t="str">
-        <v>Dev POD 4/Suraj</v>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I61" t="str">
         <v>No</v>
@@ -2171,7 +2171,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Shivam Shete</v>
+        <v>Sree Sowndarya Barani K</v>
       </c>
       <c r="B62" t="str">
         <v/>
@@ -2183,16 +2183,16 @@
         <v>Dev</v>
       </c>
       <c r="E62" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F62" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G62" t="str">
         <v/>
       </c>
       <c r="H62" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I62" t="str">
         <v>No</v>
@@ -2200,13 +2200,13 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Shivam Surendra Shete</v>
+        <v>Sridaran N M</v>
       </c>
       <c r="B63" t="str">
-        <v>shivam.surendra.shete@pwc.com</v>
+        <v/>
       </c>
       <c r="C63" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D63" t="str">
         <v>Dev</v>
@@ -2218,10 +2218,10 @@
         <v>IR4</v>
       </c>
       <c r="G63" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v/>
       </c>
       <c r="H63" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I63" t="str">
         <v>No</v>
@@ -2229,28 +2229,28 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Shravya Nanjundaswamy</v>
+        <v>Sunandha Sanda</v>
       </c>
       <c r="B64" t="str">
-        <v>shravya.nanjundaswamy@pwc.com</v>
+        <v/>
       </c>
       <c r="C64" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D64" t="str">
         <v>Dev</v>
       </c>
       <c r="E64" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F64" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G64" t="str">
-        <v>Outage</v>
+        <v/>
       </c>
       <c r="H64" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v/>
       </c>
       <c r="I64" t="str">
         <v>No</v>
@@ -2258,13 +2258,13 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Sree Sowndarya Barani K</v>
+        <v>Surya Teja Poka</v>
       </c>
       <c r="B65" t="str">
-        <v>sree.sowndarya.barani.k@pwc.com</v>
+        <v/>
       </c>
       <c r="C65" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D65" t="str">
         <v>Dev</v>
@@ -2276,10 +2276,10 @@
         <v>IR4</v>
       </c>
       <c r="G65" t="str">
-        <v>Case Management</v>
+        <v/>
       </c>
       <c r="H65" t="str">
-        <v>Case Management POD</v>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I65" t="str">
         <v>No</v>
@@ -2287,13 +2287,13 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Sridaran N M</v>
+        <v>Venkata Sai Harika Ambati</v>
       </c>
       <c r="B66" t="str">
-        <v/>
+        <v>venkata.sai.harika.ambati@pwc.com</v>
       </c>
       <c r="C66" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D66" t="str">
         <v>Dev</v>
@@ -2305,10 +2305,10 @@
         <v>IR4</v>
       </c>
       <c r="G66" t="str">
-        <v/>
+        <v>Energy Management</v>
       </c>
       <c r="H66" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I66" t="str">
         <v>No</v>
@@ -2316,28 +2316,28 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Sridaran Natarajan Muralidharan</v>
+        <v>Aditya Talwar</v>
       </c>
       <c r="B67" t="str">
-        <v>sridaran.n.m@pwc.com</v>
+        <v>aditya.talwar@pwc.com</v>
       </c>
       <c r="C67" t="str">
-        <v>Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D67" t="str">
-        <v>Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E67" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F67" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G67" t="str">
-        <v>Multi Move In/Transfer/Amend</v>
+        <v>Account Maintenance | Customer ID &amp; Fraud</v>
       </c>
       <c r="H67" t="str">
-        <v/>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I67" t="str">
         <v>No</v>
@@ -2345,16 +2345,16 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Surya Teja Poka</v>
+        <v>Anurag Jakkal</v>
       </c>
       <c r="B68" t="str">
-        <v>poka.suryateja@pwc.com</v>
+        <v>jakkal.anurag.surendra@pwc.com</v>
       </c>
       <c r="C68" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D68" t="str">
-        <v>Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E68" t="str">
         <v>IR4</v>
@@ -2363,10 +2363,10 @@
         <v>IR4</v>
       </c>
       <c r="G68" t="str">
-        <v>Outage</v>
+        <v>Energy Management</v>
       </c>
       <c r="H68" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I68" t="str">
         <v>No</v>
@@ -2374,28 +2374,28 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Venkata Sai Harika Ambati</v>
+        <v>Pornima Rajguru</v>
       </c>
       <c r="B69" t="str">
-        <v/>
+        <v>Poornima.atul.rajguru@pwc.com</v>
       </c>
       <c r="C69" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D69" t="str">
-        <v>Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E69" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="F69" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="G69" t="str">
-        <v/>
+        <v>Outage</v>
       </c>
       <c r="H69" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I69" t="str">
         <v>No</v>
@@ -2403,10 +2403,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Aditya Talwar</v>
+        <v>Rinky Chawla</v>
       </c>
       <c r="B70" t="str">
-        <v>aditya.talwar@pwc.com</v>
+        <v>rinky.chawla@pwc.com</v>
       </c>
       <c r="C70" t="str">
         <v>Manager</v>
@@ -2421,10 +2421,10 @@
         <v>IR3.2/IR4</v>
       </c>
       <c r="G70" t="str">
-        <v>Account Maintenance | Customer ID &amp; Fraud</v>
+        <v>Case Management</v>
       </c>
       <c r="H70" t="str">
-        <v>Dev POD 6/Aditya</v>
+        <v>Case Management POD</v>
       </c>
       <c r="I70" t="str">
         <v>No</v>
@@ -2432,10 +2432,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Anurag Jakkal</v>
+        <v>Shreya LNU</v>
       </c>
       <c r="B71" t="str">
-        <v>jakkal.anurag.surendra@pwc.com</v>
+        <v>shreya.l.lnu@pwc.com</v>
       </c>
       <c r="C71" t="str">
         <v>Manager</v>
@@ -2444,16 +2444,16 @@
         <v>Dev Lead</v>
       </c>
       <c r="E71" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F71" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G71" t="str">
-        <v>Energy Management</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H71" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v>Dev POD 1/Shreya</v>
       </c>
       <c r="I71" t="str">
         <v>No</v>
@@ -2461,28 +2461,28 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Jason Pereira</v>
+        <v>Sneha Girigoudar</v>
       </c>
       <c r="B72" t="str">
-        <v>jason.c.pereira@pwc.com</v>
+        <v>sneha.raosaheb.girigoudar@pwc.com</v>
       </c>
       <c r="C72" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D72" t="str">
         <v>Dev Lead</v>
       </c>
       <c r="E72" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F72" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G72" t="str">
-        <v>Multi Move In/Transfer/Amend</v>
+        <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
       </c>
       <c r="H72" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I72" t="str">
         <v>No</v>
@@ -2490,28 +2490,28 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Niket Saxena</v>
+        <v>Suraj Ghodmare</v>
       </c>
       <c r="B73" t="str">
-        <v>niket.saxena@pwc.com</v>
+        <v>suraj.ghodmare@pwc.com</v>
       </c>
       <c r="C73" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D73" t="str">
         <v>Dev Lead</v>
       </c>
       <c r="E73" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F73" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G73" t="str">
-        <v>Field Management</v>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H73" t="str">
-        <v>Field Management POD</v>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I73" t="str">
         <v>No</v>
@@ -2519,28 +2519,28 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Pornima Rajguru</v>
+        <v>B Rajkumar</v>
       </c>
       <c r="B74" t="str">
-        <v>Poornima.atul.rajguru@pwc.com</v>
+        <v/>
       </c>
       <c r="C74" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D74" t="str">
-        <v>Dev Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E74" t="str">
-        <v>IR3.X</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F74" t="str">
-        <v>IR3.X</v>
+        <v>All</v>
       </c>
       <c r="G74" t="str">
-        <v>Outage</v>
+        <v>DevOps</v>
       </c>
       <c r="H74" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v/>
       </c>
       <c r="I74" t="str">
         <v>No</v>
@@ -2548,28 +2548,28 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Rinky Chawla</v>
+        <v>Rhitik Khanna</v>
       </c>
       <c r="B75" t="str">
-        <v>rinky.chawla@pwc.com</v>
+        <v>rhitik.khanna@pwc.com</v>
       </c>
       <c r="C75" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D75" t="str">
-        <v>Dev Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E75" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F75" t="str">
-        <v>IR3.2/IR4</v>
+        <v>All</v>
       </c>
       <c r="G75" t="str">
-        <v>Case Management</v>
+        <v>DevOps</v>
       </c>
       <c r="H75" t="str">
-        <v>Case Management POD</v>
+        <v/>
       </c>
       <c r="I75" t="str">
         <v>No</v>
@@ -2577,28 +2577,28 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Shreya LNU</v>
+        <v>Santosh Kumar Jangam</v>
       </c>
       <c r="B76" t="str">
-        <v>shreya.l.lnu@pwc.com</v>
+        <v>santosh.kumar.jangam@pwc.com</v>
       </c>
       <c r="C76" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D76" t="str">
-        <v>Dev Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E76" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F76" t="str">
-        <v>IR3.2/IR4</v>
+        <v>All</v>
       </c>
       <c r="G76" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>DevOps</v>
       </c>
       <c r="H76" t="str">
-        <v>Dev POD 1/Shreya</v>
+        <v/>
       </c>
       <c r="I76" t="str">
         <v>No</v>
@@ -2606,28 +2606,28 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Sneha Girigoudar</v>
+        <v>Shatakshi Srivastava</v>
       </c>
       <c r="B77" t="str">
-        <v>sneha.raosaheb.girigoudar@pwc.com</v>
+        <v>shatakshi.s.srivastava@pwc.com</v>
       </c>
       <c r="C77" t="str">
         <v>Manager</v>
       </c>
       <c r="D77" t="str">
-        <v>Dev Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E77" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F77" t="str">
-        <v>IR3.2/IR4</v>
+        <v>All</v>
       </c>
       <c r="G77" t="str">
-        <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
+        <v>DevOps</v>
       </c>
       <c r="H77" t="str">
-        <v>Dev POD 2/Sneha G</v>
+        <v/>
       </c>
       <c r="I77" t="str">
         <v>No</v>
@@ -2635,28 +2635,28 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Suraj Ghodmare</v>
+        <v>Vinay Vadrevu</v>
       </c>
       <c r="B78" t="str">
-        <v>suraj.ghodmare@pwc.com</v>
+        <v/>
       </c>
       <c r="C78" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D78" t="str">
-        <v>Dev Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E78" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F78" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G78" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>DevOps</v>
       </c>
       <c r="H78" t="str">
-        <v>Dev POD 4/Suraj</v>
+        <v/>
       </c>
       <c r="I78" t="str">
         <v>No</v>
@@ -2664,28 +2664,28 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Sweta Sharma</v>
+        <v>Ritesh Nanda</v>
       </c>
       <c r="B79" t="str">
-        <v>sweta.s.sharma@pwc.com</v>
+        <v>ritesh.nanda@pwc.com</v>
       </c>
       <c r="C79" t="str">
         <v>Manager</v>
       </c>
       <c r="D79" t="str">
-        <v>Dev Lead</v>
+        <v>DevOps Lead</v>
       </c>
       <c r="E79" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F79" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G79" t="str">
-        <v>Outage</v>
+        <v>DevOps</v>
       </c>
       <c r="H79" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v/>
       </c>
       <c r="I79" t="str">
         <v>No</v>
@@ -2693,22 +2693,22 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>B Rajkumar</v>
+        <v>Shabnam Nasreen</v>
       </c>
       <c r="B80" t="str">
-        <v>b.rajkumar@pwc.com</v>
+        <v>shabnam.nasreen@pwc.com</v>
       </c>
       <c r="C80" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D80" t="str">
-        <v>DevOps</v>
+        <v>DevOps Lead</v>
       </c>
       <c r="E80" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F80" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G80" t="str">
         <v>DevOps</v>
@@ -2722,25 +2722,25 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Rhitik Khanna</v>
+        <v>Anto Germans</v>
       </c>
       <c r="B81" t="str">
-        <v>rhitik.khanna@pwc.com</v>
+        <v>anto.a.germans@pwc.com</v>
       </c>
       <c r="C81" t="str">
-        <v>Senior Associate</v>
+        <v>Director</v>
       </c>
       <c r="D81" t="str">
-        <v>DevOps</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E81" t="str">
-        <v>Cross-Functional</v>
+        <v>Leadership</v>
       </c>
       <c r="F81" t="str">
         <v>All</v>
       </c>
       <c r="G81" t="str">
-        <v>DevOps</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H81" t="str">
         <v/>
@@ -2751,25 +2751,25 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Rodolfo Duarte</v>
+        <v>Matthew Rupas</v>
       </c>
       <c r="B82" t="str">
-        <v>rodolfo.d.duarte@pwc.com</v>
+        <v>matthew.i.rupas@pwc.com</v>
       </c>
       <c r="C82" t="str">
-        <v>Administrative</v>
+        <v>Partner</v>
       </c>
       <c r="D82" t="str">
-        <v>DevOps</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E82" t="str">
-        <v>IR4</v>
+        <v>Leadership</v>
       </c>
       <c r="F82" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G82" t="str">
-        <v>DevOps</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H82" t="str">
         <v/>
@@ -2780,25 +2780,25 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Santosh Kumar Jangam</v>
+        <v>Sujith Pillai</v>
       </c>
       <c r="B83" t="str">
-        <v>santosh.kumar.jangam@pwc.com</v>
+        <v>sujith.s.pillai@pwc.com</v>
       </c>
       <c r="C83" t="str">
-        <v>Senior Associate</v>
+        <v>Director</v>
       </c>
       <c r="D83" t="str">
-        <v>DevOps</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E83" t="str">
-        <v>Cross-Functional</v>
+        <v>Leadership</v>
       </c>
       <c r="F83" t="str">
         <v>All</v>
       </c>
       <c r="G83" t="str">
-        <v>DevOps</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H83" t="str">
         <v/>
@@ -2809,25 +2809,25 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Shatakshi Srivastava</v>
+        <v>Ted Capaldi</v>
       </c>
       <c r="B84" t="str">
-        <v>shatakshi.s.srivastava@pwc.com</v>
+        <v>theodore.capaldi@pwc.com</v>
       </c>
       <c r="C84" t="str">
-        <v>Manager</v>
+        <v>Partner</v>
       </c>
       <c r="D84" t="str">
-        <v>DevOps</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E84" t="str">
-        <v>Cross-Functional</v>
+        <v>Leadership</v>
       </c>
       <c r="F84" t="str">
         <v>All</v>
       </c>
       <c r="G84" t="str">
-        <v>DevOps</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H84" t="str">
         <v/>
@@ -2838,16 +2838,16 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Vinay Vadrevu</v>
+        <v>Pranav Singh</v>
       </c>
       <c r="B85" t="str">
-        <v/>
+        <v>pranav.s.singh@pwc.com</v>
       </c>
       <c r="C85" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D85" t="str">
-        <v>DevOps</v>
+        <v>Integration Dev</v>
       </c>
       <c r="E85" t="str">
         <v>Cross-Functional</v>
@@ -2856,7 +2856,7 @@
         <v>All</v>
       </c>
       <c r="G85" t="str">
-        <v>DevOps</v>
+        <v>Integration</v>
       </c>
       <c r="H85" t="str">
         <v/>
@@ -2867,16 +2867,16 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Ritesh Nanda</v>
+        <v>Vasudha Tandon</v>
       </c>
       <c r="B86" t="str">
-        <v>ritesh.nanda@pwc.com</v>
+        <v>vasudha.tandon@pwc.com</v>
       </c>
       <c r="C86" t="str">
         <v>Manager</v>
       </c>
       <c r="D86" t="str">
-        <v>DevOps Lead</v>
+        <v>Integration Dev</v>
       </c>
       <c r="E86" t="str">
         <v>Cross-Functional</v>
@@ -2885,7 +2885,7 @@
         <v>All</v>
       </c>
       <c r="G86" t="str">
-        <v>DevOps</v>
+        <v>Integration</v>
       </c>
       <c r="H86" t="str">
         <v/>
@@ -2896,16 +2896,16 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Shabnam Nasreen</v>
+        <v>Arun Kumar Krishnareddy Obannareddy</v>
       </c>
       <c r="B87" t="str">
-        <v>shabnam.nasreen@pwc.com</v>
+        <v>arun.kumar.krishnareddy.obannareddy@pwc.com</v>
       </c>
       <c r="C87" t="str">
         <v>Manager</v>
       </c>
       <c r="D87" t="str">
-        <v>DevOps Lead</v>
+        <v>Integration Lead</v>
       </c>
       <c r="E87" t="str">
         <v>Cross-Functional</v>
@@ -2914,7 +2914,7 @@
         <v>All</v>
       </c>
       <c r="G87" t="str">
-        <v>DevOps</v>
+        <v>Integration</v>
       </c>
       <c r="H87" t="str">
         <v/>
@@ -2925,25 +2925,25 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Anto Germans</v>
+        <v>Kodi Elangovan</v>
       </c>
       <c r="B88" t="str">
-        <v>anto.a.germans@pwc.com</v>
+        <v>kodiyarasan.elangovan@pwc.com</v>
       </c>
       <c r="C88" t="str">
-        <v>Director</v>
+        <v>Manager</v>
       </c>
       <c r="D88" t="str">
-        <v>Engagement Lead</v>
+        <v>Integration Lead</v>
       </c>
       <c r="E88" t="str">
-        <v>Leadership</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F88" t="str">
         <v>All</v>
       </c>
       <c r="G88" t="str">
-        <v>Program Leadership</v>
+        <v>Integration</v>
       </c>
       <c r="H88" t="str">
         <v/>
@@ -2954,25 +2954,25 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Matthew Rupas</v>
+        <v>Adithya Sankar S</v>
       </c>
       <c r="B89" t="str">
-        <v>matthew.i.rupas@pwc.com</v>
+        <v/>
       </c>
       <c r="C89" t="str">
-        <v>Partner</v>
+        <v/>
       </c>
       <c r="D89" t="str">
-        <v>Engagement Lead</v>
+        <v>Intern</v>
       </c>
       <c r="E89" t="str">
-        <v>Leadership</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F89" t="str">
         <v>All</v>
       </c>
       <c r="G89" t="str">
-        <v>Program Leadership</v>
+        <v/>
       </c>
       <c r="H89" t="str">
         <v/>
@@ -2983,25 +2983,25 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Sujith Pillai</v>
+        <v>Kishor S</v>
       </c>
       <c r="B90" t="str">
-        <v>sujith.s.pillai@pwc.com</v>
+        <v/>
       </c>
       <c r="C90" t="str">
-        <v>Director</v>
+        <v/>
       </c>
       <c r="D90" t="str">
-        <v>Engagement Lead</v>
+        <v>Intern</v>
       </c>
       <c r="E90" t="str">
-        <v>Leadership</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F90" t="str">
         <v>All</v>
       </c>
       <c r="G90" t="str">
-        <v>Program Leadership</v>
+        <v/>
       </c>
       <c r="H90" t="str">
         <v/>
@@ -3012,25 +3012,25 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Ted Capaldi</v>
+        <v>Krithika Harishchandra Shettigar</v>
       </c>
       <c r="B91" t="str">
-        <v>theodore.capaldi@pwc.com</v>
+        <v/>
       </c>
       <c r="C91" t="str">
-        <v>Partner</v>
+        <v/>
       </c>
       <c r="D91" t="str">
-        <v>Engagement Lead</v>
+        <v>Intern</v>
       </c>
       <c r="E91" t="str">
-        <v>Leadership</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F91" t="str">
         <v>All</v>
       </c>
       <c r="G91" t="str">
-        <v>Program Leadership</v>
+        <v/>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -3041,16 +3041,16 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Pranav Singh</v>
+        <v>Potumanchi Sree Yashana</v>
       </c>
       <c r="B92" t="str">
-        <v>pranav.s.singh@pwc.com</v>
+        <v/>
       </c>
       <c r="C92" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D92" t="str">
-        <v>Integration Dev</v>
+        <v>Intern</v>
       </c>
       <c r="E92" t="str">
         <v>Cross-Functional</v>
@@ -3059,7 +3059,7 @@
         <v>All</v>
       </c>
       <c r="G92" t="str">
-        <v>Integration</v>
+        <v/>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -3070,16 +3070,16 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Vasudha Tandon</v>
+        <v>Ziyad Auti</v>
       </c>
       <c r="B93" t="str">
-        <v>vasudha.tandon@pwc.com</v>
+        <v/>
       </c>
       <c r="C93" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D93" t="str">
-        <v>Integration Dev</v>
+        <v>Intern</v>
       </c>
       <c r="E93" t="str">
         <v>Cross-Functional</v>
@@ -3088,7 +3088,7 @@
         <v>All</v>
       </c>
       <c r="G93" t="str">
-        <v>Integration</v>
+        <v/>
       </c>
       <c r="H93" t="str">
         <v/>
@@ -3099,28 +3099,28 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Arun Kumar Krishnareddy Obannareddy</v>
+        <v>Jason Pereira</v>
       </c>
       <c r="B94" t="str">
-        <v>arun.kumar.krishnareddy.obannareddy@pwc.com</v>
+        <v/>
       </c>
       <c r="C94" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D94" t="str">
-        <v>Integration Lead</v>
+        <v>Lead</v>
       </c>
       <c r="E94" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F94" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G94" t="str">
-        <v>Integration</v>
+        <v/>
       </c>
       <c r="H94" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I94" t="str">
         <v>No</v>
@@ -3128,28 +3128,28 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Kodi Elangovan</v>
+        <v>Niket Saxena</v>
       </c>
       <c r="B95" t="str">
-        <v>kodiyarasan.elangovan@pwc.com</v>
+        <v/>
       </c>
       <c r="C95" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D95" t="str">
-        <v>Integration Lead</v>
+        <v>Lead</v>
       </c>
       <c r="E95" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F95" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G95" t="str">
-        <v>Integration</v>
+        <v/>
       </c>
       <c r="H95" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I95" t="str">
         <v>No</v>
@@ -3157,28 +3157,28 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Adithya Sankar S</v>
+        <v>Sweta Sharma</v>
       </c>
       <c r="B96" t="str">
-        <v>adithya.sankar@pwc.com</v>
+        <v/>
       </c>
       <c r="C96" t="str">
-        <v>Intern</v>
+        <v/>
       </c>
       <c r="D96" t="str">
-        <v>Intern</v>
+        <v>Lead</v>
       </c>
       <c r="E96" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F96" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G96" t="str">
-        <v>Interns</v>
+        <v/>
       </c>
       <c r="H96" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I96" t="str">
         <v>No</v>
@@ -3186,28 +3186,28 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Kishor S</v>
+        <v>Mayur Kinhekar</v>
       </c>
       <c r="B97" t="str">
-        <v>kishor.s@pwc.com</v>
+        <v>mayur.murlidhar.kinhekar@pwc.com</v>
       </c>
       <c r="C97" t="str">
-        <v>Intern</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D97" t="str">
-        <v>Intern</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E97" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.X</v>
       </c>
       <c r="F97" t="str">
-        <v>All</v>
+        <v>IR3.X/IR4</v>
       </c>
       <c r="G97" t="str">
-        <v>Interns</v>
+        <v>Outage</v>
       </c>
       <c r="H97" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I97" t="str">
         <v>No</v>
@@ -3215,25 +3215,25 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Krithika Harishchandra Shettigar</v>
+        <v>Namrata Uttareshwar Bansode</v>
       </c>
       <c r="B98" t="str">
-        <v>krithika.shettigar@pwc.com</v>
+        <v>namrata.uttareshwar.bansode@pwc.com</v>
       </c>
       <c r="C98" t="str">
-        <v>Intern</v>
+        <v>Manager</v>
       </c>
       <c r="D98" t="str">
-        <v>Intern</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E98" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F98" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G98" t="str">
-        <v>Interns</v>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H98" t="str">
         <v/>
@@ -3244,28 +3244,28 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Potumanchi Sree Yashana</v>
+        <v>Parul Prasad</v>
       </c>
       <c r="B99" t="str">
-        <v>potumanchi.yashana@pwc.com</v>
+        <v>parul.prasad@pwc.com</v>
       </c>
       <c r="C99" t="str">
-        <v>Intern</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D99" t="str">
-        <v>Intern</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E99" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F99" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G99" t="str">
-        <v>Interns</v>
+        <v>Energy Management</v>
       </c>
       <c r="H99" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I99" t="str">
         <v>No</v>
@@ -3273,28 +3273,28 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Ziyad Auti</v>
+        <v>Akhil Palakeel</v>
       </c>
       <c r="B100" t="str">
-        <v>ziyad.auti@pwc.com</v>
+        <v/>
       </c>
       <c r="C100" t="str">
-        <v>Intern</v>
+        <v/>
       </c>
       <c r="D100" t="str">
-        <v>Intern</v>
+        <v>Offshore Solution Analyst</v>
       </c>
       <c r="E100" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F100" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G100" t="str">
-        <v>Interns</v>
+        <v/>
       </c>
       <c r="H100" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I100" t="str">
         <v>No</v>
@@ -3302,25 +3302,25 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Akhil J Palakeel</v>
+        <v>Namrata Bansode</v>
       </c>
       <c r="B101" t="str">
-        <v>akhil.j.palakeel@pwc.com</v>
+        <v/>
       </c>
       <c r="C101" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D101" t="str">
-        <v>Offshore SA</v>
+        <v>Offshore Solution Analyst</v>
       </c>
       <c r="E101" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F101" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G101" t="str">
-        <v>Multi Move In/Transfer/Amend</v>
+        <v/>
       </c>
       <c r="H101" t="str">
         <v/>
@@ -3331,28 +3331,28 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Mayur Kinhekar</v>
+        <v>Prayas Abinash</v>
       </c>
       <c r="B102" t="str">
-        <v>mayur.murlidhar.kinhekar@pwc.com</v>
+        <v/>
       </c>
       <c r="C102" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D102" t="str">
-        <v>Offshore SA</v>
+        <v>Offshore Solution Analyst</v>
       </c>
       <c r="E102" t="str">
-        <v>IR3.X</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F102" t="str">
-        <v>IR3.X/IR4</v>
+        <v>All</v>
       </c>
       <c r="G102" t="str">
-        <v>Outage</v>
+        <v/>
       </c>
       <c r="H102" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v/>
       </c>
       <c r="I102" t="str">
         <v>No</v>
@@ -3360,28 +3360,28 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>Namrata Uttareshwar Bansode</v>
+        <v>Cicily Deng</v>
       </c>
       <c r="B103" t="str">
-        <v>namrata.uttareshwar.bansode@pwc.com</v>
+        <v>cicily.deng@pwc.com</v>
       </c>
       <c r="C103" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D103" t="str">
-        <v>Offshore SA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E103" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F103" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G103" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v>Case Management</v>
       </c>
       <c r="H103" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I103" t="str">
         <v>No</v>
@@ -3389,28 +3389,28 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>Parul Prasad</v>
+        <v>Deneys Van Der Merwe</v>
       </c>
       <c r="B104" t="str">
-        <v>parul.prasad@pwc.com</v>
+        <v>deneys.van.der.merwe@pwc.com</v>
       </c>
       <c r="C104" t="str">
         <v>Associate</v>
       </c>
       <c r="D104" t="str">
-        <v>Offshore SA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E104" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F104" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G104" t="str">
-        <v>Energy Management</v>
+        <v>Case Management</v>
       </c>
       <c r="H104" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v>Case Management POD</v>
       </c>
       <c r="I104" t="str">
         <v>No</v>
@@ -3418,28 +3418,28 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>Prayas Abinash</v>
+        <v>Gianna Caruso</v>
       </c>
       <c r="B105" t="str">
-        <v>prayas.abinash@pwc.com</v>
+        <v>gianna.caruso@pwc.com</v>
       </c>
       <c r="C105" t="str">
         <v>Associate</v>
       </c>
       <c r="D105" t="str">
-        <v>Offshore SA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E105" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F105" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G105" t="str">
-        <v>Account Maintenance</v>
+        <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H105" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I105" t="str">
         <v>No</v>
@@ -3447,28 +3447,28 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>Akhil Palakeel</v>
+        <v>Jitain Mohun</v>
       </c>
       <c r="B106" t="str">
         <v/>
       </c>
       <c r="C106" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D106" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E106" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="F106" t="str">
-        <v>IR4</v>
+        <v>IR3.X/IR4</v>
       </c>
       <c r="G106" t="str">
-        <v/>
+        <v>Outage</v>
       </c>
       <c r="H106" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I106" t="str">
         <v>No</v>
@@ -3476,28 +3476,28 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>Namrata Bansode</v>
+        <v>Michael O'shea</v>
       </c>
       <c r="B107" t="str">
-        <v/>
+        <v>michael.o.oshea@pwc.com</v>
       </c>
       <c r="C107" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D107" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E107" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F107" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G107" t="str">
-        <v/>
+        <v>Interactions/Search</v>
       </c>
       <c r="H107" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I107" t="str">
         <v>No</v>
@@ -3505,10 +3505,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Cicily Deng</v>
+        <v>Rohan Bandla</v>
       </c>
       <c r="B108" t="str">
-        <v>cicily.deng@pwc.com</v>
+        <v/>
       </c>
       <c r="C108" t="str">
         <v>Senior Associate</v>
@@ -3517,16 +3517,16 @@
         <v>Onshore SA</v>
       </c>
       <c r="E108" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F108" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G108" t="str">
-        <v>Case Management</v>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H108" t="str">
-        <v>Case Management POD</v>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I108" t="str">
         <v>No</v>
@@ -3534,28 +3534,28 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Deneys Van Der Merwe</v>
+        <v>Sahithi Manne</v>
       </c>
       <c r="B109" t="str">
-        <v>deneys.van.der.merwe@pwc.com</v>
+        <v/>
       </c>
       <c r="C109" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D109" t="str">
         <v>Onshore SA</v>
       </c>
       <c r="E109" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F109" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G109" t="str">
-        <v>Case Management</v>
+        <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
       </c>
       <c r="H109" t="str">
-        <v>Case Management POD</v>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I109" t="str">
         <v>No</v>
@@ -3563,28 +3563,28 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Gianna Caruso</v>
+        <v>Russell Stein</v>
       </c>
       <c r="B110" t="str">
-        <v>gianna.caruso@pwc.com</v>
+        <v/>
       </c>
       <c r="C110" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D110" t="str">
-        <v>Onshore SA</v>
+        <v>Onshore Solution Analyst</v>
       </c>
       <c r="E110" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F110" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G110" t="str">
-        <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
+        <v>Billing &amp; Usage</v>
       </c>
       <c r="H110" t="str">
-        <v>Dev POD 4/Suraj</v>
+        <v>Dev POD 1/Shreya</v>
       </c>
       <c r="I110" t="str">
         <v>No</v>
@@ -3592,28 +3592,28 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Jitain Mohun</v>
+        <v>Courtney Hawkins</v>
       </c>
       <c r="B111" t="str">
-        <v/>
+        <v>courtney.c.hawkins@pwc.com</v>
       </c>
       <c r="C111" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D111" t="str">
-        <v>Onshore SA</v>
+        <v>PMO</v>
       </c>
       <c r="E111" t="str">
-        <v>IR3.X</v>
+        <v>Leadership</v>
       </c>
       <c r="F111" t="str">
-        <v>IR3.X/IR4</v>
+        <v>All</v>
       </c>
       <c r="G111" t="str">
-        <v>Outage</v>
+        <v>PMO</v>
       </c>
       <c r="H111" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v/>
       </c>
       <c r="I111" t="str">
         <v>No</v>
@@ -3621,28 +3621,28 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Michael O'shea</v>
+        <v>Paarth Sonwaney</v>
       </c>
       <c r="B112" t="str">
-        <v>michael.o.oshea@pwc.com</v>
+        <v>paarth.sonwaney@pwc.com</v>
       </c>
       <c r="C112" t="str">
-        <v>Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D112" t="str">
-        <v>Onshore SA</v>
+        <v>PMO</v>
       </c>
       <c r="E112" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F112" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G112" t="str">
-        <v>Interactions/Search</v>
+        <v>PMO</v>
       </c>
       <c r="H112" t="str">
-        <v>Dev POD 2/Sneha G</v>
+        <v/>
       </c>
       <c r="I112" t="str">
         <v>No</v>
@@ -3650,28 +3650,28 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>Rohan Bandla</v>
+        <v>Shanta Samlal</v>
       </c>
       <c r="B113" t="str">
-        <v/>
+        <v>shanta.samlal@pwc.com</v>
       </c>
       <c r="C113" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D113" t="str">
-        <v>Onshore SA</v>
+        <v>PMO</v>
       </c>
       <c r="E113" t="str">
-        <v>IR4</v>
+        <v>Leadership</v>
       </c>
       <c r="F113" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G113" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>PMO</v>
       </c>
       <c r="H113" t="str">
-        <v>Dev POD 2/Sneha G</v>
+        <v/>
       </c>
       <c r="I113" t="str">
         <v>No</v>
@@ -3679,28 +3679,28 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>Russell Stein</v>
+        <v>Aakanksha</v>
       </c>
       <c r="B114" t="str">
-        <v>russell.stein@pwc.com</v>
+        <v/>
       </c>
       <c r="C114" t="str">
-        <v>Senior Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D114" t="str">
-        <v>Onshore SA</v>
+        <v>QA</v>
       </c>
       <c r="E114" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="F114" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="G114" t="str">
-        <v>Billing &amp; Usage</v>
+        <v>Outage</v>
       </c>
       <c r="H114" t="str">
-        <v>Dev POD 1/Shreya</v>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I114" t="str">
         <v>No</v>
@@ -3708,28 +3708,28 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>Sahithi Manne</v>
+        <v>Argene Francisco</v>
       </c>
       <c r="B115" t="str">
         <v/>
       </c>
       <c r="C115" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D115" t="str">
-        <v>Onshore SA</v>
+        <v>QA</v>
       </c>
       <c r="E115" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F115" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G115" t="str">
-        <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
+        <v>Move In, Transfer</v>
       </c>
       <c r="H115" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I115" t="str">
         <v>No</v>
@@ -3737,25 +3737,25 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>Courtney Hawkins</v>
+        <v>Argene M. Francisco</v>
       </c>
       <c r="B116" t="str">
-        <v>courtney.c.hawkins@pwc.com</v>
+        <v>argene.francisco@pwc.com</v>
       </c>
       <c r="C116" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D116" t="str">
-        <v>PMO</v>
+        <v>QA</v>
       </c>
       <c r="E116" t="str">
-        <v>Leadership</v>
+        <v>IR3.2</v>
       </c>
       <c r="F116" t="str">
         <v>All</v>
       </c>
       <c r="G116" t="str">
-        <v>PMO</v>
+        <v>Move In/Transfer</v>
       </c>
       <c r="H116" t="str">
         <v/>
@@ -3766,28 +3766,28 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>Paarth Sonwaney</v>
+        <v>Ashit Prashant Golwala</v>
       </c>
       <c r="B117" t="str">
-        <v>paarth.sonwaney@pwc.com</v>
+        <v>ashit.prashant.golwala@pwc.com</v>
       </c>
       <c r="C117" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D117" t="str">
-        <v>PMO</v>
+        <v>QA</v>
       </c>
       <c r="E117" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F117" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G117" t="str">
-        <v>PMO</v>
+        <v>Energy Management</v>
       </c>
       <c r="H117" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I117" t="str">
         <v>No</v>
@@ -3795,25 +3795,25 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Shanta Samlal</v>
+        <v>Bhyravabhotla Naga Lakshmi Sirisha</v>
       </c>
       <c r="B118" t="str">
-        <v>shanta.samlal@pwc.com</v>
+        <v>bhyravabhotla.naga.lakshmi.sirisha@pwc.com</v>
       </c>
       <c r="C118" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D118" t="str">
-        <v>PMO</v>
+        <v>QA</v>
       </c>
       <c r="E118" t="str">
-        <v>Leadership</v>
+        <v>IR3.2</v>
       </c>
       <c r="F118" t="str">
         <v>All</v>
       </c>
       <c r="G118" t="str">
-        <v>PMO</v>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H118" t="str">
         <v/>
@@ -3824,7 +3824,7 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Aakanksha</v>
+        <v>Diksha</v>
       </c>
       <c r="B119" t="str">
         <v/>
@@ -3853,7 +3853,7 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Argene Francisco</v>
+        <v>Dnyanesh Prakash Painjan</v>
       </c>
       <c r="B120" t="str">
         <v/>
@@ -3882,13 +3882,13 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Argene M. Francisco</v>
+        <v>Dnyanesh Prakash Painjane</v>
       </c>
       <c r="B121" t="str">
-        <v>argene.francisco@pwc.com</v>
+        <v>dnyanesh.prakash.painjane@pwc.com</v>
       </c>
       <c r="C121" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D121" t="str">
         <v>QA</v>
@@ -3911,25 +3911,25 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Ashit Golwala</v>
+        <v>Girlee Alvarado</v>
       </c>
       <c r="B122" t="str">
-        <v>ashit.prashant.golwala@pwc.com</v>
+        <v/>
       </c>
       <c r="C122" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D122" t="str">
         <v>QA</v>
       </c>
       <c r="E122" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F122" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G122" t="str">
-        <v>Energy Management</v>
+        <v>Move Out, Transfer</v>
       </c>
       <c r="H122" t="str">
         <v/>
@@ -3940,28 +3940,28 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>Ashit Prashant Golwala</v>
+        <v>Girlee P. Alvarado</v>
       </c>
       <c r="B123" t="str">
-        <v/>
+        <v>girlee.alvarado@pwc.com</v>
       </c>
       <c r="C123" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D123" t="str">
         <v>QA</v>
       </c>
       <c r="E123" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F123" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G123" t="str">
-        <v/>
+        <v>Move Out/Transfer</v>
       </c>
       <c r="H123" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I123" t="str">
         <v>No</v>
@@ -3969,25 +3969,25 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>Bhyravabhotla Naga Lakshmi Sirisha</v>
+        <v>Grace Nazareno</v>
       </c>
       <c r="B124" t="str">
-        <v>bhyravabhotla.naga.lakshmi.sirisha@pwc.com</v>
+        <v/>
       </c>
       <c r="C124" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D124" t="str">
         <v>QA</v>
       </c>
       <c r="E124" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F124" t="str">
         <v>All</v>
       </c>
       <c r="G124" t="str">
-        <v>Move In/Move Out</v>
+        <v>Payment &amp; Payment Options, Billing Programs</v>
       </c>
       <c r="H124" t="str">
         <v/>
@@ -3998,28 +3998,28 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>Diksha</v>
+        <v>ISH Jacinto</v>
       </c>
       <c r="B125" t="str">
         <v/>
       </c>
       <c r="C125" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D125" t="str">
         <v>QA</v>
       </c>
       <c r="E125" t="str">
-        <v>IR3.X</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F125" t="str">
-        <v>IR3.X</v>
+        <v>All</v>
       </c>
       <c r="G125" t="str">
-        <v>Outage</v>
+        <v>Move Out</v>
       </c>
       <c r="H125" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v/>
       </c>
       <c r="I125" t="str">
         <v>No</v>
@@ -4027,25 +4027,25 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>Dnyanesh Prakash Painjan</v>
+        <v>Israel L. Jacinto</v>
       </c>
       <c r="B126" t="str">
-        <v/>
+        <v>israel.jacinto@pwc.com</v>
       </c>
       <c r="C126" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D126" t="str">
         <v>QA</v>
       </c>
       <c r="E126" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F126" t="str">
         <v>All</v>
       </c>
       <c r="G126" t="str">
-        <v>Move In, Transfer</v>
+        <v>Move Out</v>
       </c>
       <c r="H126" t="str">
         <v/>
@@ -4056,13 +4056,13 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>Dnyanesh Prakash Painjane</v>
+        <v>Keerthana Manjunath</v>
       </c>
       <c r="B127" t="str">
-        <v>dnyanesh.prakash.painjane@pwc.com</v>
+        <v/>
       </c>
       <c r="C127" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D127" t="str">
         <v>QA</v>
@@ -4074,7 +4074,7 @@
         <v>All</v>
       </c>
       <c r="G127" t="str">
-        <v>Move In/Transfer</v>
+        <v>Transfer</v>
       </c>
       <c r="H127" t="str">
         <v/>
@@ -4085,28 +4085,28 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>Girlee Alvarado</v>
+        <v>Lokesh Sai</v>
       </c>
       <c r="B128" t="str">
-        <v/>
+        <v>lokesh.sai@pwc.com</v>
       </c>
       <c r="C128" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D128" t="str">
         <v>QA</v>
       </c>
       <c r="E128" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F128" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G128" t="str">
-        <v>Move Out, Transfer</v>
+        <v>Energy Management</v>
       </c>
       <c r="H128" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I128" t="str">
         <v>No</v>
@@ -4114,13 +4114,13 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>Girlee P. Alvarado</v>
+        <v>Maneesha</v>
       </c>
       <c r="B129" t="str">
-        <v>girlee.alvarado@pwc.com</v>
+        <v/>
       </c>
       <c r="C129" t="str">
-        <v>Senior Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D129" t="str">
         <v>QA</v>
@@ -4132,7 +4132,7 @@
         <v>All</v>
       </c>
       <c r="G129" t="str">
-        <v>Move Out/Transfer</v>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H129" t="str">
         <v/>
@@ -4143,25 +4143,25 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Grace Nazareno</v>
+        <v>Mary Grace Carinan Nazareno</v>
       </c>
       <c r="B130" t="str">
-        <v/>
+        <v>mary.grace.nazareno@pwc.com</v>
       </c>
       <c r="C130" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D130" t="str">
         <v>QA</v>
       </c>
       <c r="E130" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F130" t="str">
         <v>All</v>
       </c>
       <c r="G130" t="str">
-        <v>Payment &amp; Payment Options, Billing Programs</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H130" t="str">
         <v/>
@@ -4172,28 +4172,28 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>ISH Jacinto</v>
+        <v>Mayand Mani</v>
       </c>
       <c r="B131" t="str">
         <v/>
       </c>
       <c r="C131" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D131" t="str">
         <v>QA</v>
       </c>
       <c r="E131" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F131" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G131" t="str">
-        <v>Move Out</v>
+        <v>Energy Management</v>
       </c>
       <c r="H131" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I131" t="str">
         <v>No</v>
@@ -4201,25 +4201,25 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>Israel L. Jacinto</v>
+        <v>Mindi Sai Bhavana</v>
       </c>
       <c r="B132" t="str">
-        <v>israel.jacinto@pwc.com</v>
+        <v/>
       </c>
       <c r="C132" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D132" t="str">
         <v>QA</v>
       </c>
       <c r="E132" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F132" t="str">
         <v>All</v>
       </c>
       <c r="G132" t="str">
-        <v>Move Out</v>
+        <v>Case Management</v>
       </c>
       <c r="H132" t="str">
         <v/>
@@ -4230,13 +4230,13 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>Keerthana Manjunath</v>
+        <v>Naga Srilekha Thummalacheruvu</v>
       </c>
       <c r="B133" t="str">
-        <v/>
+        <v>naga.t.thummalacheruvu@pwc.com</v>
       </c>
       <c r="C133" t="str">
-        <v>Infosys</v>
+        <v>Associate</v>
       </c>
       <c r="D133" t="str">
         <v>QA</v>
@@ -4248,7 +4248,7 @@
         <v>All</v>
       </c>
       <c r="G133" t="str">
-        <v>Transfer</v>
+        <v>Move In</v>
       </c>
       <c r="H133" t="str">
         <v/>
@@ -4259,28 +4259,28 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>Lokesh Sai</v>
+        <v>Nikita</v>
       </c>
       <c r="B134" t="str">
-        <v>madana.lokesh.dhana.sai@pwc.com</v>
+        <v/>
       </c>
       <c r="C134" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D134" t="str">
         <v>QA</v>
       </c>
       <c r="E134" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F134" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G134" t="str">
-        <v>Energy Management</v>
+        <v>Payment &amp; Payment Options</v>
       </c>
       <c r="H134" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I134" t="str">
         <v>No</v>
@@ -4288,7 +4288,7 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Maneesha</v>
+        <v>Nilesh</v>
       </c>
       <c r="B135" t="str">
         <v/>
@@ -4306,7 +4306,7 @@
         <v>All</v>
       </c>
       <c r="G135" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H135" t="str">
         <v/>
@@ -4317,25 +4317,25 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>Mary Grace Carinan Nazareno</v>
+        <v>Prasanna</v>
       </c>
       <c r="B136" t="str">
-        <v>mary.grace.nazareno@pwc.com</v>
+        <v/>
       </c>
       <c r="C136" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D136" t="str">
         <v>QA</v>
       </c>
       <c r="E136" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F136" t="str">
         <v>All</v>
       </c>
       <c r="G136" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Billing Programs</v>
       </c>
       <c r="H136" t="str">
         <v/>
@@ -4346,10 +4346,10 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>Mindi Sai Bhavana</v>
+        <v>Prasanna Nangnure</v>
       </c>
       <c r="B137" t="str">
-        <v>mindi.sai.bhavana@pwc.com</v>
+        <v>prasanna.y.nangnure@pwc.com</v>
       </c>
       <c r="C137" t="str">
         <v>Associate</v>
@@ -4358,13 +4358,13 @@
         <v>QA</v>
       </c>
       <c r="E137" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F137" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G137" t="str">
-        <v/>
+        <v>Billing Programs</v>
       </c>
       <c r="H137" t="str">
         <v/>
@@ -4375,13 +4375,13 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>Naga Srilekha Thummalacheruvu</v>
+        <v>Pratik Mahajan</v>
       </c>
       <c r="B138" t="str">
-        <v>naga.t.thummalacheruvu@pwc.com</v>
+        <v>pratik.sunil.mahajan@pwc.com</v>
       </c>
       <c r="C138" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D138" t="str">
         <v>QA</v>
@@ -4393,7 +4393,7 @@
         <v>All</v>
       </c>
       <c r="G138" t="str">
-        <v>Move In</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H138" t="str">
         <v/>
@@ -4404,25 +4404,25 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>Navyashree Shantharam</v>
+        <v>Pritam</v>
       </c>
       <c r="B139" t="str">
-        <v>navyashree.s.shantharam@pwc.com</v>
+        <v/>
       </c>
       <c r="C139" t="str">
-        <v>Senior Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D139" t="str">
         <v>QA</v>
       </c>
       <c r="E139" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F139" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G139" t="str">
-        <v/>
+        <v>Account Maintenance</v>
       </c>
       <c r="H139" t="str">
         <v/>
@@ -4433,13 +4433,13 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>Nikita</v>
+        <v>Raveendra Reddy</v>
       </c>
       <c r="B140" t="str">
-        <v/>
+        <v>raveendra.t.reddy@pwc.com</v>
       </c>
       <c r="C140" t="str">
-        <v>Infosys</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D140" t="str">
         <v>QA</v>
@@ -4451,7 +4451,7 @@
         <v>All</v>
       </c>
       <c r="G140" t="str">
-        <v>Payment &amp; Payment Options</v>
+        <v>Transfer</v>
       </c>
       <c r="H140" t="str">
         <v/>
@@ -4462,28 +4462,28 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>Nilesh</v>
+        <v>Sagnik Chakraborty</v>
       </c>
       <c r="B141" t="str">
-        <v/>
+        <v>sagnik.chakraborty@pwc.com</v>
       </c>
       <c r="C141" t="str">
-        <v>Infosys</v>
+        <v>Associate</v>
       </c>
       <c r="D141" t="str">
         <v>QA</v>
       </c>
       <c r="E141" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F141" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G141" t="str">
-        <v>Account Maintenance</v>
+        <v>Energy Management</v>
       </c>
       <c r="H141" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I141" t="str">
         <v>No</v>
@@ -4491,25 +4491,25 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>Prasanna</v>
+        <v>Sanjana</v>
       </c>
       <c r="B142" t="str">
         <v/>
       </c>
       <c r="C142" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D142" t="str">
         <v>QA</v>
       </c>
       <c r="E142" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F142" t="str">
         <v>All</v>
       </c>
       <c r="G142" t="str">
-        <v>Billing Programs</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H142" t="str">
         <v/>
@@ -4520,13 +4520,13 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>Prasanna Nangnure</v>
+        <v>Smita</v>
       </c>
       <c r="B143" t="str">
-        <v>prasanna.y.nangnure@pwc.com</v>
+        <v/>
       </c>
       <c r="C143" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D143" t="str">
         <v>QA</v>
@@ -4538,7 +4538,7 @@
         <v>All</v>
       </c>
       <c r="G143" t="str">
-        <v>Billing Programs</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H143" t="str">
         <v/>
@@ -4549,10 +4549,10 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>Pratik Mahajan</v>
+        <v>Sonal Yadav</v>
       </c>
       <c r="B144" t="str">
-        <v>pratik.sunil.mahajan@pwc.com</v>
+        <v>sonal.y.yadav@pwc.com</v>
       </c>
       <c r="C144" t="str">
         <v>Senior Associate</v>
@@ -4567,7 +4567,7 @@
         <v>All</v>
       </c>
       <c r="G144" t="str">
-        <v>Interactions/Search</v>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H144" t="str">
         <v/>
@@ -4578,7 +4578,7 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>Pritam</v>
+        <v>Venugopal Sinde</v>
       </c>
       <c r="B145" t="str">
         <v/>
@@ -4596,7 +4596,7 @@
         <v>All</v>
       </c>
       <c r="G145" t="str">
-        <v>Account Maintenance</v>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H145" t="str">
         <v/>
@@ -4607,25 +4607,25 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>Raveendra Reddy</v>
+        <v>Vidyashree</v>
       </c>
       <c r="B146" t="str">
-        <v>raveendra.t.reddy@pwc.com</v>
+        <v/>
       </c>
       <c r="C146" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D146" t="str">
         <v>QA</v>
       </c>
       <c r="E146" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F146" t="str">
         <v>All</v>
       </c>
       <c r="G146" t="str">
-        <v>Transfer</v>
+        <v>Payment &amp; Payment Options</v>
       </c>
       <c r="H146" t="str">
         <v/>
@@ -4636,28 +4636,28 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>Sagnik Chakraborty</v>
+        <v>Vidyashree S R</v>
       </c>
       <c r="B147" t="str">
-        <v>sagnik.c.chakraborty@pwc.com</v>
+        <v>vidyashree.s.r@pwc.com</v>
       </c>
       <c r="C147" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D147" t="str">
         <v>QA</v>
       </c>
       <c r="E147" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F147" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G147" t="str">
-        <v>Energy Management</v>
+        <v>Payment &amp; Payment Options</v>
       </c>
       <c r="H147" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I147" t="str">
         <v>No</v>
@@ -4665,16 +4665,16 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>Sanjana</v>
+        <v>Rajaraman A</v>
       </c>
       <c r="B148" t="str">
-        <v/>
+        <v>rajaraman.a@pwc.com</v>
       </c>
       <c r="C148" t="str">
-        <v>Infosys</v>
+        <v>Manager</v>
       </c>
       <c r="D148" t="str">
-        <v>QA</v>
+        <v>QA Lead</v>
       </c>
       <c r="E148" t="str">
         <v>IR3.2</v>
@@ -4683,7 +4683,7 @@
         <v>All</v>
       </c>
       <c r="G148" t="str">
-        <v>Interactions/Search</v>
+        <v>QA - All Value Streams</v>
       </c>
       <c r="H148" t="str">
         <v/>
@@ -4694,25 +4694,25 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Shreya Maji</v>
+        <v>Tyaga Pati</v>
       </c>
       <c r="B149" t="str">
-        <v>shreya.maji@pwc.com</v>
+        <v>tyaga.pati@pwc.com</v>
       </c>
       <c r="C149" t="str">
-        <v>Associate</v>
+        <v>Senior Manager</v>
       </c>
       <c r="D149" t="str">
-        <v>QA</v>
+        <v>Solution Architect</v>
       </c>
       <c r="E149" t="str">
-        <v>IR4</v>
+        <v>Leadership</v>
       </c>
       <c r="F149" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G149" t="str">
-        <v/>
+        <v>Architecture</v>
       </c>
       <c r="H149" t="str">
         <v/>
@@ -4723,25 +4723,25 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>Smita</v>
+        <v>Rodolfo Duarte</v>
       </c>
       <c r="B150" t="str">
         <v/>
       </c>
       <c r="C150" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D150" t="str">
-        <v>QA</v>
+        <v>Team</v>
       </c>
       <c r="E150" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F150" t="str">
         <v>All</v>
       </c>
       <c r="G150" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v/>
       </c>
       <c r="H150" t="str">
         <v/>
@@ -4752,25 +4752,25 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>Sonal Yadav</v>
+        <v>Hemant Jain</v>
       </c>
       <c r="B151" t="str">
-        <v>sonal.y.yadav@pwc.com</v>
+        <v>hemant.jain@pwc.com</v>
       </c>
       <c r="C151" t="str">
-        <v>Senior Associate</v>
+        <v>Senior Manager</v>
       </c>
       <c r="D151" t="str">
-        <v>QA</v>
+        <v>Technical Architect</v>
       </c>
       <c r="E151" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F151" t="str">
         <v>All</v>
       </c>
       <c r="G151" t="str">
-        <v>Move In/Move Out</v>
+        <v>Architecture</v>
       </c>
       <c r="H151" t="str">
         <v/>
@@ -4781,25 +4781,25 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>Venugopal Sinde</v>
+        <v>Harish Govindareddy</v>
       </c>
       <c r="B152" t="str">
-        <v/>
+        <v>harish.govindareddy@pwc.com</v>
       </c>
       <c r="C152" t="str">
-        <v>Infosys</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D152" t="str">
-        <v>QA</v>
+        <v>Windsurf/Performance Dev</v>
       </c>
       <c r="E152" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F152" t="str">
         <v>All</v>
       </c>
       <c r="G152" t="str">
-        <v>Move In/Move Out</v>
+        <v>Windsurf/Performance</v>
       </c>
       <c r="H152" t="str">
         <v/>
@@ -4810,16 +4810,16 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>Vidyashree</v>
+        <v>Sanket Mundargi</v>
       </c>
       <c r="B153" t="str">
-        <v/>
+        <v>sanket.mundargi@pwc.com</v>
       </c>
       <c r="C153" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D153" t="str">
-        <v>QA</v>
+        <v>Windsurf/Performance Dev</v>
       </c>
       <c r="E153" t="str">
         <v>Cross-Functional</v>
@@ -4828,192 +4828,18 @@
         <v>All</v>
       </c>
       <c r="G153" t="str">
-        <v>Payment &amp; Payment Options</v>
+        <v>Windsurf/Performance</v>
       </c>
       <c r="H153" t="str">
         <v/>
       </c>
       <c r="I153" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="str">
-        <v>Vidyashree S R</v>
-      </c>
-      <c r="B154" t="str">
-        <v>vidyashree.s.r@pwc.com</v>
-      </c>
-      <c r="C154" t="str">
-        <v>Senior Associate</v>
-      </c>
-      <c r="D154" t="str">
-        <v>QA</v>
-      </c>
-      <c r="E154" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="F154" t="str">
-        <v>All</v>
-      </c>
-      <c r="G154" t="str">
-        <v>Payment &amp; Payment Options</v>
-      </c>
-      <c r="H154" t="str">
-        <v/>
-      </c>
-      <c r="I154" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="str">
-        <v>Rajaraman A</v>
-      </c>
-      <c r="B155" t="str">
-        <v>rajaraman.a@pwc.com</v>
-      </c>
-      <c r="C155" t="str">
-        <v>Manager</v>
-      </c>
-      <c r="D155" t="str">
-        <v>QA Lead</v>
-      </c>
-      <c r="E155" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="F155" t="str">
-        <v>All</v>
-      </c>
-      <c r="G155" t="str">
-        <v>QA - All Value Streams</v>
-      </c>
-      <c r="H155" t="str">
-        <v/>
-      </c>
-      <c r="I155" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="str">
-        <v>Tyaga Pati</v>
-      </c>
-      <c r="B156" t="str">
-        <v>tyaga.pati@pwc.com</v>
-      </c>
-      <c r="C156" t="str">
-        <v>Senior Manager</v>
-      </c>
-      <c r="D156" t="str">
-        <v>Solution Architect</v>
-      </c>
-      <c r="E156" t="str">
-        <v>Leadership</v>
-      </c>
-      <c r="F156" t="str">
-        <v>All</v>
-      </c>
-      <c r="G156" t="str">
-        <v>Architecture</v>
-      </c>
-      <c r="H156" t="str">
-        <v/>
-      </c>
-      <c r="I156" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="str">
-        <v>Hemant Jain</v>
-      </c>
-      <c r="B157" t="str">
-        <v>hemant.jain@pwc.com</v>
-      </c>
-      <c r="C157" t="str">
-        <v>Senior Manager</v>
-      </c>
-      <c r="D157" t="str">
-        <v>Technical Architect</v>
-      </c>
-      <c r="E157" t="str">
-        <v>Leadership</v>
-      </c>
-      <c r="F157" t="str">
-        <v>All</v>
-      </c>
-      <c r="G157" t="str">
-        <v>Architecture</v>
-      </c>
-      <c r="H157" t="str">
-        <v/>
-      </c>
-      <c r="I157" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="str">
-        <v>Harish Govindareddy</v>
-      </c>
-      <c r="B158" t="str">
-        <v>harish.govindareddy@pwc.com</v>
-      </c>
-      <c r="C158" t="str">
-        <v>Senior Associate</v>
-      </c>
-      <c r="D158" t="str">
-        <v>Windsurf/Performance Dev</v>
-      </c>
-      <c r="E158" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F158" t="str">
-        <v>All</v>
-      </c>
-      <c r="G158" t="str">
-        <v>Windsurf/Performance</v>
-      </c>
-      <c r="H158" t="str">
-        <v/>
-      </c>
-      <c r="I158" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="str">
-        <v>Sanket Mundargi</v>
-      </c>
-      <c r="B159" t="str">
-        <v>sanket.mundargi@pwc.com</v>
-      </c>
-      <c r="C159" t="str">
-        <v>Associate</v>
-      </c>
-      <c r="D159" t="str">
-        <v>Windsurf/Performance Dev</v>
-      </c>
-      <c r="E159" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F159" t="str">
-        <v>All</v>
-      </c>
-      <c r="G159" t="str">
-        <v>Windsurf/Performance</v>
-      </c>
-      <c r="H159" t="str">
-        <v/>
-      </c>
-      <c r="I159" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I159"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I153"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Restored v215: feat: add Sunandha Sanda to staffing and team data
Added new team member Sunandha Sanda to staffing data and dev pod list
</commit_message>
<xml_diff>
--- a/public/FPL Staffing.xlsx
+++ b/public/FPL Staffing.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I153"/>
+  <dimension ref="A1:I159"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1214,13 +1214,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Ankit Mishra</v>
+        <v>Ambati Venkata Sai Harika</v>
       </c>
       <c r="B29" t="str">
-        <v>ankit.b.mishra@pwc.com</v>
+        <v>venkata.sai.harika.ambati@pwc.com</v>
       </c>
       <c r="C29" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D29" t="str">
         <v>Dev</v>
@@ -1232,7 +1232,7 @@
         <v>IR4</v>
       </c>
       <c r="G29" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Energy Management</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -1243,13 +1243,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Ankit Verma</v>
+        <v>Ankit Mishra</v>
       </c>
       <c r="B30" t="str">
-        <v/>
+        <v>ankit.b.mishra@pwc.com</v>
       </c>
       <c r="C30" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D30" t="str">
         <v>Dev</v>
@@ -1261,10 +1261,10 @@
         <v>IR4</v>
       </c>
       <c r="G30" t="str">
-        <v/>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H30" t="str">
-        <v>Case Management POD</v>
+        <v/>
       </c>
       <c r="I30" t="str">
         <v>No</v>
@@ -1272,13 +1272,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Chaitra Hanchinal</v>
+        <v>Ankit Prasad Verma</v>
       </c>
       <c r="B31" t="str">
-        <v/>
+        <v>ankit.prasad.verma@pwc.com</v>
       </c>
       <c r="C31" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D31" t="str">
         <v>Dev</v>
@@ -1290,10 +1290,10 @@
         <v>IR4</v>
       </c>
       <c r="G31" t="str">
-        <v/>
+        <v>Case Management</v>
       </c>
       <c r="H31" t="str">
-        <v>Field Management POD</v>
+        <v/>
       </c>
       <c r="I31" t="str">
         <v>No</v>
@@ -1301,13 +1301,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Cheruku Pranay Reddy</v>
+        <v>Ankit Verma</v>
       </c>
       <c r="B32" t="str">
-        <v>cheruku.pranay.reddy@pwc.com</v>
+        <v/>
       </c>
       <c r="C32" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D32" t="str">
         <v>Dev</v>
@@ -1319,10 +1319,10 @@
         <v>IR4</v>
       </c>
       <c r="G32" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v/>
       </c>
       <c r="H32" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I32" t="str">
         <v>No</v>
@@ -1330,13 +1330,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Jaya Lakshmi Papolu</v>
+        <v>Chaitra Hanchinal</v>
       </c>
       <c r="B33" t="str">
-        <v/>
+        <v>chaitra.s.hanchinal@pwc.com</v>
       </c>
       <c r="C33" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D33" t="str">
         <v>Dev</v>
@@ -1348,7 +1348,7 @@
         <v>IR4</v>
       </c>
       <c r="G33" t="str">
-        <v/>
+        <v>Field Management</v>
       </c>
       <c r="H33" t="str">
         <v>Field Management POD</v>
@@ -1359,10 +1359,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Jayoti Chatterji</v>
+        <v>Cheruku Pranay Reddy</v>
       </c>
       <c r="B34" t="str">
-        <v>jayoti.chatterji@pwc.com</v>
+        <v>cheruku.pranay.reddy@pwc.com</v>
       </c>
       <c r="C34" t="str">
         <v>Senior Associate</v>
@@ -1371,16 +1371,16 @@
         <v>Dev</v>
       </c>
       <c r="E34" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F34" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="G34" t="str">
-        <v>Outage</v>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H34" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v/>
       </c>
       <c r="I34" t="str">
         <v>No</v>
@@ -1388,13 +1388,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>John Jyothula</v>
+        <v>Jaya Lakshmi Papolu</v>
       </c>
       <c r="B35" t="str">
-        <v/>
+        <v>jaya.lakshmi.papolu@pwc.com</v>
       </c>
       <c r="C35" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D35" t="str">
         <v>Dev</v>
@@ -1406,10 +1406,10 @@
         <v>IR4</v>
       </c>
       <c r="G35" t="str">
-        <v/>
+        <v>Field Management</v>
       </c>
       <c r="H35" t="str">
-        <v>Case Management POD</v>
+        <v>Field Management POD</v>
       </c>
       <c r="I35" t="str">
         <v>No</v>
@@ -1417,28 +1417,28 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Kankshitha Yalamuru</v>
+        <v>Jayoti Chatterji</v>
       </c>
       <c r="B36" t="str">
-        <v/>
+        <v>jayoti.chatterji@pwc.com</v>
       </c>
       <c r="C36" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D36" t="str">
         <v>Dev</v>
       </c>
       <c r="E36" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.X</v>
       </c>
       <c r="F36" t="str">
-        <v>All</v>
+        <v>IR3.X</v>
       </c>
       <c r="G36" t="str">
-        <v/>
+        <v>Outage</v>
       </c>
       <c r="H36" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I36" t="str">
         <v>No</v>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Kavita Jha</v>
+        <v>John Jyothula</v>
       </c>
       <c r="B37" t="str">
         <v/>
@@ -1467,7 +1467,7 @@
         <v/>
       </c>
       <c r="H37" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v>Case Management POD</v>
       </c>
       <c r="I37" t="str">
         <v>No</v>
@@ -1475,10 +1475,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Madhumita Kodidela</v>
+        <v>Jyothula John Paramjyothi</v>
       </c>
       <c r="B38" t="str">
-        <v>madhumitha.kodidela@pwc.com</v>
+        <v>john.paramjyothi.jyothula@pwc.com</v>
       </c>
       <c r="C38" t="str">
         <v>Senior Associate</v>
@@ -1487,16 +1487,16 @@
         <v>Dev</v>
       </c>
       <c r="E38" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F38" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G38" t="str">
-        <v>Interactions/Search</v>
+        <v>Case Management</v>
       </c>
       <c r="H38" t="str">
-        <v>Dev POD 2/Sneha G</v>
+        <v/>
       </c>
       <c r="I38" t="str">
         <v>No</v>
@@ -1504,25 +1504,25 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Manu Tyagi</v>
+        <v>Kankshitha Yalamuru</v>
       </c>
       <c r="B39" t="str">
-        <v/>
+        <v>yalamuru.sai.kankshitha@pwc.com</v>
       </c>
       <c r="C39" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D39" t="str">
         <v>Dev</v>
       </c>
       <c r="E39" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F39" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G39" t="str">
-        <v/>
+        <v>Billing &amp; Usage</v>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -1533,10 +1533,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Mounika Depuri</v>
+        <v>Kavita Jha</v>
       </c>
       <c r="B40" t="str">
-        <v>mounika.depuri@pwc.com</v>
+        <v>kavita.jha@pwc.com</v>
       </c>
       <c r="C40" t="str">
         <v>Senior Associate</v>
@@ -1545,16 +1545,16 @@
         <v>Dev</v>
       </c>
       <c r="E40" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F40" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G40" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Outage</v>
       </c>
       <c r="H40" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I40" t="str">
         <v>No</v>
@@ -1562,28 +1562,28 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Mrithika Kumaresan</v>
+        <v>Madhumita Kodidela</v>
       </c>
       <c r="B41" t="str">
-        <v/>
+        <v>madhumitha.kodidela@pwc.com</v>
       </c>
       <c r="C41" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D41" t="str">
         <v>Dev</v>
       </c>
       <c r="E41" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F41" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G41" t="str">
-        <v/>
+        <v>Interactions/Search</v>
       </c>
       <c r="H41" t="str">
-        <v>Field Management POD</v>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I41" t="str">
         <v>No</v>
@@ -1591,10 +1591,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Mylavarapu V N R Saketh</v>
+        <v>Manu Tyagi</v>
       </c>
       <c r="B42" t="str">
-        <v>mylavarapu.v.n.r.saketh@pwc.com</v>
+        <v>manu.tyagi@pwc.com</v>
       </c>
       <c r="C42" t="str">
         <v>Senior Associate</v>
@@ -1609,10 +1609,10 @@
         <v>IR4</v>
       </c>
       <c r="G42" t="str">
-        <v>Energy Management</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H42" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I42" t="str">
         <v>No</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Naman Hiran</v>
+        <v>Mounika Depuri</v>
       </c>
       <c r="B43" t="str">
-        <v>naman.hiran@pwc.com</v>
+        <v>mounika.depuri@pwc.com</v>
       </c>
       <c r="C43" t="str">
         <v>Senior Associate</v>
@@ -1632,16 +1632,16 @@
         <v>Dev</v>
       </c>
       <c r="E43" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F43" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G43" t="str">
-        <v>Energy Management</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H43" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I43" t="str">
         <v>No</v>
@@ -1649,28 +1649,28 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Nishi Jain</v>
+        <v>Mrithika Kumaresan</v>
       </c>
       <c r="B44" t="str">
-        <v/>
+        <v>mrithika.kumaresan@pwc.com</v>
       </c>
       <c r="C44" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D44" t="str">
         <v>Dev</v>
       </c>
       <c r="E44" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F44" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G44" t="str">
-        <v/>
+        <v>Field Management</v>
       </c>
       <c r="H44" t="str">
-        <v>Dev POD 6/Aditya</v>
+        <v>Field Management POD</v>
       </c>
       <c r="I44" t="str">
         <v>No</v>
@@ -1678,10 +1678,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Nishi Narendra Jain</v>
+        <v>Mylavarapu V N R Saketh</v>
       </c>
       <c r="B45" t="str">
-        <v>jain.u.nishi@pwc.com</v>
+        <v>mylavarapu.v.n.r.saketh@pwc.com</v>
       </c>
       <c r="C45" t="str">
         <v>Senior Associate</v>
@@ -1690,16 +1690,16 @@
         <v>Dev</v>
       </c>
       <c r="E45" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F45" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G45" t="str">
-        <v>Account Maintenance</v>
+        <v>Energy Management</v>
       </c>
       <c r="H45" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I45" t="str">
         <v>No</v>
@@ -1707,13 +1707,13 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Nivetha Sudharsanam</v>
+        <v>Naman Hiran</v>
       </c>
       <c r="B46" t="str">
-        <v/>
+        <v xml:space="preserve">naman.h.hiran@pwc.com </v>
       </c>
       <c r="C46" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D46" t="str">
         <v>Dev</v>
@@ -1725,10 +1725,10 @@
         <v>IR4</v>
       </c>
       <c r="G46" t="str">
-        <v/>
+        <v>Energy Management</v>
       </c>
       <c r="H46" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I46" t="str">
         <v>No</v>
@@ -1736,13 +1736,13 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Piyush Singh</v>
+        <v>Nishi Jain</v>
       </c>
       <c r="B47" t="str">
-        <v>piyush.ss.singh@pwc.com</v>
+        <v/>
       </c>
       <c r="C47" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D47" t="str">
         <v>Dev</v>
@@ -1754,10 +1754,10 @@
         <v>IR3.2</v>
       </c>
       <c r="G47" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v/>
       </c>
       <c r="H47" t="str">
-        <v>Dev POD 4/Suraj</v>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I47" t="str">
         <v>No</v>
@@ -1765,28 +1765,28 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Pradeep Lambu</v>
+        <v>Nishi Narendra Jain</v>
       </c>
       <c r="B48" t="str">
-        <v/>
+        <v>jain.u.nishi@pwc.com</v>
       </c>
       <c r="C48" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D48" t="str">
         <v>Dev</v>
       </c>
       <c r="E48" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F48" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G48" t="str">
-        <v/>
+        <v>Account Maintenance</v>
       </c>
       <c r="H48" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v/>
       </c>
       <c r="I48" t="str">
         <v>No</v>
@@ -1794,28 +1794,28 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Pranay Reddy</v>
+        <v>Nivetha Sudharsanam</v>
       </c>
       <c r="B49" t="str">
-        <v/>
+        <v>nivetha.sudharsanam@pwc.com</v>
       </c>
       <c r="C49" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D49" t="str">
         <v>Dev</v>
       </c>
       <c r="E49" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F49" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G49" t="str">
-        <v/>
+        <v>Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H49" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I49" t="str">
         <v>No</v>
@@ -1823,28 +1823,28 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Prasad P</v>
+        <v>Piyush Singh</v>
       </c>
       <c r="B50" t="str">
-        <v/>
+        <v>piyush.ss.singh@pwc.com</v>
       </c>
       <c r="C50" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D50" t="str">
         <v>Dev</v>
       </c>
       <c r="E50" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F50" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G50" t="str">
-        <v/>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H50" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I50" t="str">
         <v>No</v>
@@ -1852,28 +1852,28 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Pratik Kurdukar</v>
+        <v>Pradeep L</v>
       </c>
       <c r="B51" t="str">
-        <v>pratik.k.kurdukar@pwc.com</v>
+        <v>pradeep.l@pwc.com</v>
       </c>
       <c r="C51" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D51" t="str">
         <v>Dev</v>
       </c>
       <c r="E51" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F51" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G51" t="str">
-        <v>Case Management</v>
+        <v>Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H51" t="str">
-        <v>Case Management POD</v>
+        <v/>
       </c>
       <c r="I51" t="str">
         <v>No</v>
@@ -1881,7 +1881,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Rida Maryam Mohammad</v>
+        <v>Pradeep Lambu</v>
       </c>
       <c r="B52" t="str">
         <v/>
@@ -1902,7 +1902,7 @@
         <v/>
       </c>
       <c r="H52" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I52" t="str">
         <v>No</v>
@@ -1910,25 +1910,25 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Rubasri S</v>
+        <v>Pranay Reddy</v>
       </c>
       <c r="B53" t="str">
-        <v>rubasri.x.s@pwc.com</v>
+        <v/>
       </c>
       <c r="C53" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D53" t="str">
         <v>Dev</v>
       </c>
       <c r="E53" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F53" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G53" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v/>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -1939,28 +1939,28 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Sahil Thadani</v>
+        <v>Prasad P</v>
       </c>
       <c r="B54" t="str">
-        <v/>
+        <v>prasad.p@pwc.com</v>
       </c>
       <c r="C54" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D54" t="str">
         <v>Dev</v>
       </c>
       <c r="E54" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F54" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G54" t="str">
-        <v/>
+        <v>Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H54" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I54" t="str">
         <v>No</v>
@@ -1968,28 +1968,28 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Sahithi Chebrolu</v>
+        <v>Pratik Kurdukar</v>
       </c>
       <c r="B55" t="str">
-        <v/>
+        <v>pratik.k.kurdukar@pwc.com</v>
       </c>
       <c r="C55" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D55" t="str">
         <v>Dev</v>
       </c>
       <c r="E55" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F55" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G55" t="str">
-        <v/>
+        <v>Case Management</v>
       </c>
       <c r="H55" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I55" t="str">
         <v>No</v>
@@ -1997,28 +1997,28 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Sandesh Saravanan</v>
+        <v>Rida Maryam Mohammad</v>
       </c>
       <c r="B56" t="str">
-        <v>sandesh.saravanan@pwc.com</v>
+        <v>rida.maryam.mohammad@pwc.com</v>
       </c>
       <c r="C56" t="str">
-        <v>Intern</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D56" t="str">
         <v>Dev</v>
       </c>
       <c r="E56" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F56" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G56" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Outage</v>
       </c>
       <c r="H56" t="str">
-        <v>IR3.2 Hypercare Support</v>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I56" t="str">
         <v>No</v>
@@ -2026,13 +2026,13 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Sanniboina Murali Krishna</v>
+        <v>Rubasri S</v>
       </c>
       <c r="B57" t="str">
-        <v/>
+        <v>rubasri.x.s@pwc.com</v>
       </c>
       <c r="C57" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D57" t="str">
         <v>Dev</v>
@@ -2044,10 +2044,10 @@
         <v>IR4</v>
       </c>
       <c r="G57" t="str">
-        <v/>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H57" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v/>
       </c>
       <c r="I57" t="str">
         <v>No</v>
@@ -2055,28 +2055,28 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Shikhar Sanjeev</v>
+        <v>Sahil Thadani</v>
       </c>
       <c r="B58" t="str">
-        <v>shikhar.sanjeev@pwc.com</v>
+        <v>sahil.kumar.thadani@pwc.com</v>
       </c>
       <c r="C58" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D58" t="str">
         <v>Dev</v>
       </c>
       <c r="E58" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F58" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G58" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Billing &amp; Usage</v>
       </c>
       <c r="H58" t="str">
-        <v>Dev POD 4/Suraj</v>
+        <v/>
       </c>
       <c r="I58" t="str">
         <v>No</v>
@@ -2084,28 +2084,28 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Shivam Shete</v>
+        <v>Sandesh Saravanan</v>
       </c>
       <c r="B59" t="str">
-        <v/>
+        <v>sandesh.saravanan@pwc.com</v>
       </c>
       <c r="C59" t="str">
-        <v/>
+        <v>Intern</v>
       </c>
       <c r="D59" t="str">
         <v>Dev</v>
       </c>
       <c r="E59" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F59" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G59" t="str">
-        <v/>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H59" t="str">
-        <v/>
+        <v>IR3.2 Hypercare Support</v>
       </c>
       <c r="I59" t="str">
         <v>No</v>
@@ -2113,10 +2113,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Shivam Surendra Shete</v>
+        <v>Sanniboina Murali Krishna</v>
       </c>
       <c r="B60" t="str">
-        <v>shivam.surendra.shete@pwc.com</v>
+        <v>sanniboina.murali.krishna@pwc.com</v>
       </c>
       <c r="C60" t="str">
         <v>Senior Associate</v>
@@ -2131,10 +2131,10 @@
         <v>IR4</v>
       </c>
       <c r="G60" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v>Outage</v>
       </c>
       <c r="H60" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I60" t="str">
         <v>No</v>
@@ -2142,28 +2142,28 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Shravya Nanjundaswamy</v>
+        <v>Shikhar Sanjeev</v>
       </c>
       <c r="B61" t="str">
-        <v/>
+        <v>shikhar.sanjeev@pwc.com</v>
       </c>
       <c r="C61" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D61" t="str">
         <v>Dev</v>
       </c>
       <c r="E61" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F61" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G61" t="str">
-        <v/>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H61" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I61" t="str">
         <v>No</v>
@@ -2171,7 +2171,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Sree Sowndarya Barani K</v>
+        <v>Shivam Shete</v>
       </c>
       <c r="B62" t="str">
         <v/>
@@ -2183,16 +2183,16 @@
         <v>Dev</v>
       </c>
       <c r="E62" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F62" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G62" t="str">
         <v/>
       </c>
       <c r="H62" t="str">
-        <v>Case Management POD</v>
+        <v/>
       </c>
       <c r="I62" t="str">
         <v>No</v>
@@ -2200,13 +2200,13 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Sridaran N M</v>
+        <v>Shivam Surendra Shete</v>
       </c>
       <c r="B63" t="str">
-        <v/>
+        <v>shivam.surendra.shete@pwc.com</v>
       </c>
       <c r="C63" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D63" t="str">
         <v>Dev</v>
@@ -2218,10 +2218,10 @@
         <v>IR4</v>
       </c>
       <c r="G63" t="str">
-        <v/>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H63" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v/>
       </c>
       <c r="I63" t="str">
         <v>No</v>
@@ -2229,28 +2229,28 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Sunandha Sanda</v>
+        <v>Shravya Nanjundaswamy</v>
       </c>
       <c r="B64" t="str">
-        <v/>
+        <v>shravya.nanjundaswamy@pwc.com</v>
       </c>
       <c r="C64" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D64" t="str">
         <v>Dev</v>
       </c>
       <c r="E64" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F64" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G64" t="str">
-        <v/>
+        <v>Outage</v>
       </c>
       <c r="H64" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I64" t="str">
         <v>No</v>
@@ -2258,13 +2258,13 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Surya Teja Poka</v>
+        <v>Sree Sowndarya Barani K</v>
       </c>
       <c r="B65" t="str">
-        <v/>
+        <v>sree.sowndarya.barani.k@pwc.com</v>
       </c>
       <c r="C65" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D65" t="str">
         <v>Dev</v>
@@ -2276,10 +2276,10 @@
         <v>IR4</v>
       </c>
       <c r="G65" t="str">
-        <v/>
+        <v>Case Management</v>
       </c>
       <c r="H65" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v>Case Management POD</v>
       </c>
       <c r="I65" t="str">
         <v>No</v>
@@ -2287,13 +2287,13 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Venkata Sai Harika Ambati</v>
+        <v>Sridaran N M</v>
       </c>
       <c r="B66" t="str">
-        <v>venkata.sai.harika.ambati@pwc.com</v>
+        <v/>
       </c>
       <c r="C66" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D66" t="str">
         <v>Dev</v>
@@ -2305,10 +2305,10 @@
         <v>IR4</v>
       </c>
       <c r="G66" t="str">
-        <v>Energy Management</v>
+        <v/>
       </c>
       <c r="H66" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I66" t="str">
         <v>No</v>
@@ -2316,28 +2316,28 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Aditya Talwar</v>
+        <v>Sridaran Natarajan Muralidharan</v>
       </c>
       <c r="B67" t="str">
-        <v>aditya.talwar@pwc.com</v>
+        <v>sridaran.n.m@pwc.com</v>
       </c>
       <c r="C67" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D67" t="str">
-        <v>Dev Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E67" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F67" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G67" t="str">
-        <v>Account Maintenance | Customer ID &amp; Fraud</v>
+        <v>Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H67" t="str">
-        <v>Dev POD 6/Aditya</v>
+        <v/>
       </c>
       <c r="I67" t="str">
         <v>No</v>
@@ -2345,16 +2345,16 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Anurag Jakkal</v>
+        <v>Surya Teja Poka</v>
       </c>
       <c r="B68" t="str">
-        <v>jakkal.anurag.surendra@pwc.com</v>
+        <v>poka.suryateja@pwc.com</v>
       </c>
       <c r="C68" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D68" t="str">
-        <v>Dev Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E68" t="str">
         <v>IR4</v>
@@ -2363,10 +2363,10 @@
         <v>IR4</v>
       </c>
       <c r="G68" t="str">
-        <v>Energy Management</v>
+        <v>Outage</v>
       </c>
       <c r="H68" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I68" t="str">
         <v>No</v>
@@ -2374,28 +2374,28 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Pornima Rajguru</v>
+        <v>Venkata Sai Harika Ambati</v>
       </c>
       <c r="B69" t="str">
-        <v>Poornima.atul.rajguru@pwc.com</v>
+        <v/>
       </c>
       <c r="C69" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D69" t="str">
-        <v>Dev Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E69" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F69" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="G69" t="str">
-        <v>Outage</v>
+        <v/>
       </c>
       <c r="H69" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I69" t="str">
         <v>No</v>
@@ -2403,10 +2403,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Rinky Chawla</v>
+        <v>Aditya Talwar</v>
       </c>
       <c r="B70" t="str">
-        <v>rinky.chawla@pwc.com</v>
+        <v>aditya.talwar@pwc.com</v>
       </c>
       <c r="C70" t="str">
         <v>Manager</v>
@@ -2421,10 +2421,10 @@
         <v>IR3.2/IR4</v>
       </c>
       <c r="G70" t="str">
-        <v>Case Management</v>
+        <v>Account Maintenance | Customer ID &amp; Fraud</v>
       </c>
       <c r="H70" t="str">
-        <v>Case Management POD</v>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I70" t="str">
         <v>No</v>
@@ -2432,10 +2432,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Shreya LNU</v>
+        <v>Anurag Jakkal</v>
       </c>
       <c r="B71" t="str">
-        <v>shreya.l.lnu@pwc.com</v>
+        <v>jakkal.anurag.surendra@pwc.com</v>
       </c>
       <c r="C71" t="str">
         <v>Manager</v>
@@ -2444,16 +2444,16 @@
         <v>Dev Lead</v>
       </c>
       <c r="E71" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F71" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G71" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Energy Management</v>
       </c>
       <c r="H71" t="str">
-        <v>Dev POD 1/Shreya</v>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I71" t="str">
         <v>No</v>
@@ -2461,28 +2461,28 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Sneha Girigoudar</v>
+        <v>Jason Pereira</v>
       </c>
       <c r="B72" t="str">
-        <v>sneha.raosaheb.girigoudar@pwc.com</v>
+        <v>jason.c.pereira@pwc.com</v>
       </c>
       <c r="C72" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D72" t="str">
         <v>Dev Lead</v>
       </c>
       <c r="E72" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F72" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G72" t="str">
-        <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
+        <v>Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H72" t="str">
-        <v>Dev POD 2/Sneha G</v>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I72" t="str">
         <v>No</v>
@@ -2490,28 +2490,28 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Suraj Ghodmare</v>
+        <v>Niket Saxena</v>
       </c>
       <c r="B73" t="str">
-        <v>suraj.ghodmare@pwc.com</v>
+        <v>niket.saxena@pwc.com</v>
       </c>
       <c r="C73" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D73" t="str">
         <v>Dev Lead</v>
       </c>
       <c r="E73" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F73" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G73" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Field Management</v>
       </c>
       <c r="H73" t="str">
-        <v>Dev POD 4/Suraj</v>
+        <v>Field Management POD</v>
       </c>
       <c r="I73" t="str">
         <v>No</v>
@@ -2519,28 +2519,28 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>B Rajkumar</v>
+        <v>Pornima Rajguru</v>
       </c>
       <c r="B74" t="str">
-        <v/>
+        <v>Poornima.atul.rajguru@pwc.com</v>
       </c>
       <c r="C74" t="str">
-        <v>Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D74" t="str">
-        <v>DevOps</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E74" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.X</v>
       </c>
       <c r="F74" t="str">
-        <v>All</v>
+        <v>IR3.X</v>
       </c>
       <c r="G74" t="str">
-        <v>DevOps</v>
+        <v>Outage</v>
       </c>
       <c r="H74" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I74" t="str">
         <v>No</v>
@@ -2548,28 +2548,28 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Rhitik Khanna</v>
+        <v>Rinky Chawla</v>
       </c>
       <c r="B75" t="str">
-        <v>rhitik.khanna@pwc.com</v>
+        <v>rinky.chawla@pwc.com</v>
       </c>
       <c r="C75" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D75" t="str">
-        <v>DevOps</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E75" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F75" t="str">
-        <v>All</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G75" t="str">
-        <v>DevOps</v>
+        <v>Case Management</v>
       </c>
       <c r="H75" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I75" t="str">
         <v>No</v>
@@ -2577,28 +2577,28 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Santosh Kumar Jangam</v>
+        <v>Shreya LNU</v>
       </c>
       <c r="B76" t="str">
-        <v>santosh.kumar.jangam@pwc.com</v>
+        <v>shreya.l.lnu@pwc.com</v>
       </c>
       <c r="C76" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D76" t="str">
-        <v>DevOps</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E76" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F76" t="str">
-        <v>All</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G76" t="str">
-        <v>DevOps</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H76" t="str">
-        <v/>
+        <v>Dev POD 1/Shreya</v>
       </c>
       <c r="I76" t="str">
         <v>No</v>
@@ -2606,28 +2606,28 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Shatakshi Srivastava</v>
+        <v>Sneha Girigoudar</v>
       </c>
       <c r="B77" t="str">
-        <v>shatakshi.s.srivastava@pwc.com</v>
+        <v>sneha.raosaheb.girigoudar@pwc.com</v>
       </c>
       <c r="C77" t="str">
         <v>Manager</v>
       </c>
       <c r="D77" t="str">
-        <v>DevOps</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E77" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F77" t="str">
-        <v>All</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G77" t="str">
-        <v>DevOps</v>
+        <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
       </c>
       <c r="H77" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I77" t="str">
         <v>No</v>
@@ -2635,28 +2635,28 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Vinay Vadrevu</v>
+        <v>Suraj Ghodmare</v>
       </c>
       <c r="B78" t="str">
-        <v/>
+        <v>suraj.ghodmare@pwc.com</v>
       </c>
       <c r="C78" t="str">
-        <v>Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D78" t="str">
-        <v>DevOps</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E78" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F78" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G78" t="str">
-        <v>DevOps</v>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H78" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I78" t="str">
         <v>No</v>
@@ -2664,28 +2664,28 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Ritesh Nanda</v>
+        <v>Sweta Sharma</v>
       </c>
       <c r="B79" t="str">
-        <v>ritesh.nanda@pwc.com</v>
+        <v>sweta.s.sharma@pwc.com</v>
       </c>
       <c r="C79" t="str">
         <v>Manager</v>
       </c>
       <c r="D79" t="str">
-        <v>DevOps Lead</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E79" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F79" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G79" t="str">
-        <v>DevOps</v>
+        <v>Outage</v>
       </c>
       <c r="H79" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I79" t="str">
         <v>No</v>
@@ -2693,22 +2693,22 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Shabnam Nasreen</v>
+        <v>B Rajkumar</v>
       </c>
       <c r="B80" t="str">
-        <v>shabnam.nasreen@pwc.com</v>
+        <v>b.rajkumar@pwc.com</v>
       </c>
       <c r="C80" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D80" t="str">
-        <v>DevOps Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E80" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F80" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G80" t="str">
         <v>DevOps</v>
@@ -2722,25 +2722,25 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Anto Germans</v>
+        <v>Rhitik Khanna</v>
       </c>
       <c r="B81" t="str">
-        <v>anto.a.germans@pwc.com</v>
+        <v>rhitik.khanna@pwc.com</v>
       </c>
       <c r="C81" t="str">
-        <v>Director</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D81" t="str">
-        <v>Engagement Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E81" t="str">
-        <v>Leadership</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F81" t="str">
         <v>All</v>
       </c>
       <c r="G81" t="str">
-        <v>Program Leadership</v>
+        <v>DevOps</v>
       </c>
       <c r="H81" t="str">
         <v/>
@@ -2751,25 +2751,25 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Matthew Rupas</v>
+        <v>Rodolfo Duarte</v>
       </c>
       <c r="B82" t="str">
-        <v>matthew.i.rupas@pwc.com</v>
+        <v>rodolfo.d.duarte@pwc.com</v>
       </c>
       <c r="C82" t="str">
-        <v>Partner</v>
+        <v>Administrative</v>
       </c>
       <c r="D82" t="str">
-        <v>Engagement Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E82" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F82" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G82" t="str">
-        <v>Program Leadership</v>
+        <v>DevOps</v>
       </c>
       <c r="H82" t="str">
         <v/>
@@ -2780,25 +2780,25 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Sujith Pillai</v>
+        <v>Santosh Kumar Jangam</v>
       </c>
       <c r="B83" t="str">
-        <v>sujith.s.pillai@pwc.com</v>
+        <v>santosh.kumar.jangam@pwc.com</v>
       </c>
       <c r="C83" t="str">
-        <v>Director</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D83" t="str">
-        <v>Engagement Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E83" t="str">
-        <v>Leadership</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F83" t="str">
         <v>All</v>
       </c>
       <c r="G83" t="str">
-        <v>Program Leadership</v>
+        <v>DevOps</v>
       </c>
       <c r="H83" t="str">
         <v/>
@@ -2809,25 +2809,25 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Ted Capaldi</v>
+        <v>Shatakshi Srivastava</v>
       </c>
       <c r="B84" t="str">
-        <v>theodore.capaldi@pwc.com</v>
+        <v>shatakshi.s.srivastava@pwc.com</v>
       </c>
       <c r="C84" t="str">
-        <v>Partner</v>
+        <v>Manager</v>
       </c>
       <c r="D84" t="str">
-        <v>Engagement Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E84" t="str">
-        <v>Leadership</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F84" t="str">
         <v>All</v>
       </c>
       <c r="G84" t="str">
-        <v>Program Leadership</v>
+        <v>DevOps</v>
       </c>
       <c r="H84" t="str">
         <v/>
@@ -2838,16 +2838,16 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Pranav Singh</v>
+        <v>Vinay Vadrevu</v>
       </c>
       <c r="B85" t="str">
-        <v>pranav.s.singh@pwc.com</v>
+        <v/>
       </c>
       <c r="C85" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D85" t="str">
-        <v>Integration Dev</v>
+        <v>DevOps</v>
       </c>
       <c r="E85" t="str">
         <v>Cross-Functional</v>
@@ -2856,7 +2856,7 @@
         <v>All</v>
       </c>
       <c r="G85" t="str">
-        <v>Integration</v>
+        <v>DevOps</v>
       </c>
       <c r="H85" t="str">
         <v/>
@@ -2867,16 +2867,16 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Vasudha Tandon</v>
+        <v>Ritesh Nanda</v>
       </c>
       <c r="B86" t="str">
-        <v>vasudha.tandon@pwc.com</v>
+        <v>ritesh.nanda@pwc.com</v>
       </c>
       <c r="C86" t="str">
         <v>Manager</v>
       </c>
       <c r="D86" t="str">
-        <v>Integration Dev</v>
+        <v>DevOps Lead</v>
       </c>
       <c r="E86" t="str">
         <v>Cross-Functional</v>
@@ -2885,7 +2885,7 @@
         <v>All</v>
       </c>
       <c r="G86" t="str">
-        <v>Integration</v>
+        <v>DevOps</v>
       </c>
       <c r="H86" t="str">
         <v/>
@@ -2896,16 +2896,16 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Arun Kumar Krishnareddy Obannareddy</v>
+        <v>Shabnam Nasreen</v>
       </c>
       <c r="B87" t="str">
-        <v>arun.kumar.krishnareddy.obannareddy@pwc.com</v>
+        <v>shabnam.nasreen@pwc.com</v>
       </c>
       <c r="C87" t="str">
         <v>Manager</v>
       </c>
       <c r="D87" t="str">
-        <v>Integration Lead</v>
+        <v>DevOps Lead</v>
       </c>
       <c r="E87" t="str">
         <v>Cross-Functional</v>
@@ -2914,7 +2914,7 @@
         <v>All</v>
       </c>
       <c r="G87" t="str">
-        <v>Integration</v>
+        <v>DevOps</v>
       </c>
       <c r="H87" t="str">
         <v/>
@@ -2925,25 +2925,25 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Kodi Elangovan</v>
+        <v>Anto Germans</v>
       </c>
       <c r="B88" t="str">
-        <v>kodiyarasan.elangovan@pwc.com</v>
+        <v>anto.a.germans@pwc.com</v>
       </c>
       <c r="C88" t="str">
-        <v>Manager</v>
+        <v>Director</v>
       </c>
       <c r="D88" t="str">
-        <v>Integration Lead</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E88" t="str">
-        <v>Cross-Functional</v>
+        <v>Leadership</v>
       </c>
       <c r="F88" t="str">
         <v>All</v>
       </c>
       <c r="G88" t="str">
-        <v>Integration</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H88" t="str">
         <v/>
@@ -2954,25 +2954,25 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Adithya Sankar S</v>
+        <v>Matthew Rupas</v>
       </c>
       <c r="B89" t="str">
-        <v/>
+        <v>matthew.i.rupas@pwc.com</v>
       </c>
       <c r="C89" t="str">
-        <v/>
+        <v>Partner</v>
       </c>
       <c r="D89" t="str">
-        <v>Intern</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E89" t="str">
-        <v>Cross-Functional</v>
+        <v>Leadership</v>
       </c>
       <c r="F89" t="str">
         <v>All</v>
       </c>
       <c r="G89" t="str">
-        <v/>
+        <v>Program Leadership</v>
       </c>
       <c r="H89" t="str">
         <v/>
@@ -2983,25 +2983,25 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Kishor S</v>
+        <v>Sujith Pillai</v>
       </c>
       <c r="B90" t="str">
-        <v/>
+        <v>sujith.s.pillai@pwc.com</v>
       </c>
       <c r="C90" t="str">
-        <v/>
+        <v>Director</v>
       </c>
       <c r="D90" t="str">
-        <v>Intern</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E90" t="str">
-        <v>Cross-Functional</v>
+        <v>Leadership</v>
       </c>
       <c r="F90" t="str">
         <v>All</v>
       </c>
       <c r="G90" t="str">
-        <v/>
+        <v>Program Leadership</v>
       </c>
       <c r="H90" t="str">
         <v/>
@@ -3012,25 +3012,25 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Krithika Harishchandra Shettigar</v>
+        <v>Ted Capaldi</v>
       </c>
       <c r="B91" t="str">
-        <v/>
+        <v>theodore.capaldi@pwc.com</v>
       </c>
       <c r="C91" t="str">
-        <v/>
+        <v>Partner</v>
       </c>
       <c r="D91" t="str">
-        <v>Intern</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E91" t="str">
-        <v>Cross-Functional</v>
+        <v>Leadership</v>
       </c>
       <c r="F91" t="str">
         <v>All</v>
       </c>
       <c r="G91" t="str">
-        <v/>
+        <v>Program Leadership</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -3041,16 +3041,16 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Potumanchi Sree Yashana</v>
+        <v>Pranav Singh</v>
       </c>
       <c r="B92" t="str">
-        <v/>
+        <v>pranav.s.singh@pwc.com</v>
       </c>
       <c r="C92" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D92" t="str">
-        <v>Intern</v>
+        <v>Integration Dev</v>
       </c>
       <c r="E92" t="str">
         <v>Cross-Functional</v>
@@ -3059,7 +3059,7 @@
         <v>All</v>
       </c>
       <c r="G92" t="str">
-        <v/>
+        <v>Integration</v>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -3070,16 +3070,16 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Ziyad Auti</v>
+        <v>Vasudha Tandon</v>
       </c>
       <c r="B93" t="str">
-        <v/>
+        <v>vasudha.tandon@pwc.com</v>
       </c>
       <c r="C93" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D93" t="str">
-        <v>Intern</v>
+        <v>Integration Dev</v>
       </c>
       <c r="E93" t="str">
         <v>Cross-Functional</v>
@@ -3088,7 +3088,7 @@
         <v>All</v>
       </c>
       <c r="G93" t="str">
-        <v/>
+        <v>Integration</v>
       </c>
       <c r="H93" t="str">
         <v/>
@@ -3099,28 +3099,28 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Jason Pereira</v>
+        <v>Arun Kumar Krishnareddy Obannareddy</v>
       </c>
       <c r="B94" t="str">
-        <v/>
+        <v>arun.kumar.krishnareddy.obannareddy@pwc.com</v>
       </c>
       <c r="C94" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D94" t="str">
-        <v>Lead</v>
+        <v>Integration Lead</v>
       </c>
       <c r="E94" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F94" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G94" t="str">
-        <v/>
+        <v>Integration</v>
       </c>
       <c r="H94" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v/>
       </c>
       <c r="I94" t="str">
         <v>No</v>
@@ -3128,28 +3128,28 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Niket Saxena</v>
+        <v>Kodi Elangovan</v>
       </c>
       <c r="B95" t="str">
-        <v/>
+        <v>kodiyarasan.elangovan@pwc.com</v>
       </c>
       <c r="C95" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D95" t="str">
-        <v>Lead</v>
+        <v>Integration Lead</v>
       </c>
       <c r="E95" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F95" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G95" t="str">
-        <v/>
+        <v>Integration</v>
       </c>
       <c r="H95" t="str">
-        <v>Field Management POD</v>
+        <v/>
       </c>
       <c r="I95" t="str">
         <v>No</v>
@@ -3157,28 +3157,28 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Sweta Sharma</v>
+        <v>Adithya Sankar S</v>
       </c>
       <c r="B96" t="str">
-        <v/>
+        <v>adithya.sankar@pwc.com</v>
       </c>
       <c r="C96" t="str">
-        <v/>
+        <v>Intern</v>
       </c>
       <c r="D96" t="str">
-        <v>Lead</v>
+        <v>Intern</v>
       </c>
       <c r="E96" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F96" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G96" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="H96" t="str">
-        <v>Dev POD 5/Sweta</v>
+        <v/>
       </c>
       <c r="I96" t="str">
         <v>No</v>
@@ -3186,28 +3186,28 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Mayur Kinhekar</v>
+        <v>Kishor S</v>
       </c>
       <c r="B97" t="str">
-        <v>mayur.murlidhar.kinhekar@pwc.com</v>
+        <v>kishor.s@pwc.com</v>
       </c>
       <c r="C97" t="str">
-        <v>Senior Associate</v>
+        <v>Intern</v>
       </c>
       <c r="D97" t="str">
-        <v>Offshore SA</v>
+        <v>Intern</v>
       </c>
       <c r="E97" t="str">
-        <v>IR3.X</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F97" t="str">
-        <v>IR3.X/IR4</v>
+        <v>All</v>
       </c>
       <c r="G97" t="str">
-        <v>Outage</v>
+        <v>Interns</v>
       </c>
       <c r="H97" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v/>
       </c>
       <c r="I97" t="str">
         <v>No</v>
@@ -3215,25 +3215,25 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Namrata Uttareshwar Bansode</v>
+        <v>Krithika Harishchandra Shettigar</v>
       </c>
       <c r="B98" t="str">
-        <v>namrata.uttareshwar.bansode@pwc.com</v>
+        <v>krithika.shettigar@pwc.com</v>
       </c>
       <c r="C98" t="str">
-        <v>Manager</v>
+        <v>Intern</v>
       </c>
       <c r="D98" t="str">
-        <v>Offshore SA</v>
+        <v>Intern</v>
       </c>
       <c r="E98" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F98" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G98" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v>Interns</v>
       </c>
       <c r="H98" t="str">
         <v/>
@@ -3244,28 +3244,28 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Parul Prasad</v>
+        <v>Potumanchi Sree Yashana</v>
       </c>
       <c r="B99" t="str">
-        <v>parul.prasad@pwc.com</v>
+        <v>potumanchi.yashana@pwc.com</v>
       </c>
       <c r="C99" t="str">
-        <v>Senior Associate</v>
+        <v>Intern</v>
       </c>
       <c r="D99" t="str">
-        <v>Offshore SA</v>
+        <v>Intern</v>
       </c>
       <c r="E99" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F99" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G99" t="str">
-        <v>Energy Management</v>
+        <v>Interns</v>
       </c>
       <c r="H99" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I99" t="str">
         <v>No</v>
@@ -3273,28 +3273,28 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Akhil Palakeel</v>
+        <v>Ziyad Auti</v>
       </c>
       <c r="B100" t="str">
-        <v/>
+        <v>ziyad.auti@pwc.com</v>
       </c>
       <c r="C100" t="str">
-        <v/>
+        <v>Intern</v>
       </c>
       <c r="D100" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>Intern</v>
       </c>
       <c r="E100" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F100" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G100" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="H100" t="str">
-        <v>Dev POD 4/Jason</v>
+        <v/>
       </c>
       <c r="I100" t="str">
         <v>No</v>
@@ -3302,25 +3302,25 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Namrata Bansode</v>
+        <v>Akhil J Palakeel</v>
       </c>
       <c r="B101" t="str">
-        <v/>
+        <v>akhil.j.palakeel@pwc.com</v>
       </c>
       <c r="C101" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D101" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E101" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F101" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G101" t="str">
-        <v/>
+        <v>Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H101" t="str">
         <v/>
@@ -3331,28 +3331,28 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Prayas Abinash</v>
+        <v>Mayur Kinhekar</v>
       </c>
       <c r="B102" t="str">
-        <v/>
+        <v>mayur.murlidhar.kinhekar@pwc.com</v>
       </c>
       <c r="C102" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D102" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E102" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.X</v>
       </c>
       <c r="F102" t="str">
-        <v>All</v>
+        <v>IR3.X/IR4</v>
       </c>
       <c r="G102" t="str">
-        <v/>
+        <v>Outage</v>
       </c>
       <c r="H102" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I102" t="str">
         <v>No</v>
@@ -3360,28 +3360,28 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>Cicily Deng</v>
+        <v>Namrata Uttareshwar Bansode</v>
       </c>
       <c r="B103" t="str">
-        <v>cicily.deng@pwc.com</v>
+        <v>namrata.uttareshwar.bansode@pwc.com</v>
       </c>
       <c r="C103" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D103" t="str">
-        <v>Onshore SA</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E103" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F103" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G103" t="str">
-        <v>Case Management</v>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H103" t="str">
-        <v>Case Management POD</v>
+        <v/>
       </c>
       <c r="I103" t="str">
         <v>No</v>
@@ -3389,28 +3389,28 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>Deneys Van Der Merwe</v>
+        <v>Parul Prasad</v>
       </c>
       <c r="B104" t="str">
-        <v>deneys.van.der.merwe@pwc.com</v>
+        <v>parul.prasad@pwc.com</v>
       </c>
       <c r="C104" t="str">
         <v>Associate</v>
       </c>
       <c r="D104" t="str">
-        <v>Onshore SA</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E104" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F104" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G104" t="str">
-        <v>Case Management</v>
+        <v>Energy Management</v>
       </c>
       <c r="H104" t="str">
-        <v>Case Management POD</v>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I104" t="str">
         <v>No</v>
@@ -3418,28 +3418,28 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>Gianna Caruso</v>
+        <v>Prayas Abinash</v>
       </c>
       <c r="B105" t="str">
-        <v>gianna.caruso@pwc.com</v>
+        <v>prayas.abinash@pwc.com</v>
       </c>
       <c r="C105" t="str">
         <v>Associate</v>
       </c>
       <c r="D105" t="str">
-        <v>Onshore SA</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E105" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F105" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G105" t="str">
-        <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H105" t="str">
-        <v>Dev POD 4/Suraj</v>
+        <v/>
       </c>
       <c r="I105" t="str">
         <v>No</v>
@@ -3447,28 +3447,28 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>Jitain Mohun</v>
+        <v>Akhil Palakeel</v>
       </c>
       <c r="B106" t="str">
         <v/>
       </c>
       <c r="C106" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D106" t="str">
-        <v>Onshore SA</v>
+        <v>Offshore Solution Analyst</v>
       </c>
       <c r="E106" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F106" t="str">
-        <v>IR3.X/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G106" t="str">
-        <v>Outage</v>
+        <v/>
       </c>
       <c r="H106" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I106" t="str">
         <v>No</v>
@@ -3476,28 +3476,28 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>Michael O'shea</v>
+        <v>Namrata Bansode</v>
       </c>
       <c r="B107" t="str">
-        <v>michael.o.oshea@pwc.com</v>
+        <v/>
       </c>
       <c r="C107" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D107" t="str">
-        <v>Onshore SA</v>
+        <v>Offshore Solution Analyst</v>
       </c>
       <c r="E107" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F107" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G107" t="str">
-        <v>Interactions/Search</v>
+        <v/>
       </c>
       <c r="H107" t="str">
-        <v>Dev POD 2/Sneha G</v>
+        <v/>
       </c>
       <c r="I107" t="str">
         <v>No</v>
@@ -3505,10 +3505,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Rohan Bandla</v>
+        <v>Cicily Deng</v>
       </c>
       <c r="B108" t="str">
-        <v/>
+        <v>cicily.deng@pwc.com</v>
       </c>
       <c r="C108" t="str">
         <v>Senior Associate</v>
@@ -3517,16 +3517,16 @@
         <v>Onshore SA</v>
       </c>
       <c r="E108" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F108" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G108" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Case Management</v>
       </c>
       <c r="H108" t="str">
-        <v>Dev POD 2/Sneha G</v>
+        <v>Case Management POD</v>
       </c>
       <c r="I108" t="str">
         <v>No</v>
@@ -3534,28 +3534,28 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Sahithi Manne</v>
+        <v>Deneys Van Der Merwe</v>
       </c>
       <c r="B109" t="str">
-        <v/>
+        <v>deneys.van.der.merwe@pwc.com</v>
       </c>
       <c r="C109" t="str">
-        <v>Infosys</v>
+        <v>Associate</v>
       </c>
       <c r="D109" t="str">
         <v>Onshore SA</v>
       </c>
       <c r="E109" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F109" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G109" t="str">
-        <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
+        <v>Case Management</v>
       </c>
       <c r="H109" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v>Case Management POD</v>
       </c>
       <c r="I109" t="str">
         <v>No</v>
@@ -3563,28 +3563,28 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Russell Stein</v>
+        <v>Gianna Caruso</v>
       </c>
       <c r="B110" t="str">
-        <v/>
+        <v>gianna.caruso@pwc.com</v>
       </c>
       <c r="C110" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D110" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E110" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F110" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G110" t="str">
-        <v>Billing &amp; Usage</v>
+        <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H110" t="str">
-        <v>Dev POD 1/Shreya</v>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I110" t="str">
         <v>No</v>
@@ -3592,28 +3592,28 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Courtney Hawkins</v>
+        <v>Jitain Mohun</v>
       </c>
       <c r="B111" t="str">
-        <v>courtney.c.hawkins@pwc.com</v>
+        <v/>
       </c>
       <c r="C111" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D111" t="str">
-        <v>PMO</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E111" t="str">
-        <v>Leadership</v>
+        <v>IR3.X</v>
       </c>
       <c r="F111" t="str">
-        <v>All</v>
+        <v>IR3.X/IR4</v>
       </c>
       <c r="G111" t="str">
-        <v>PMO</v>
+        <v>Outage</v>
       </c>
       <c r="H111" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I111" t="str">
         <v>No</v>
@@ -3621,28 +3621,28 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Paarth Sonwaney</v>
+        <v>Michael O'shea</v>
       </c>
       <c r="B112" t="str">
-        <v>paarth.sonwaney@pwc.com</v>
+        <v>michael.o.oshea@pwc.com</v>
       </c>
       <c r="C112" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D112" t="str">
-        <v>PMO</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E112" t="str">
-        <v>Leadership</v>
+        <v>IR3.2</v>
       </c>
       <c r="F112" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G112" t="str">
-        <v>PMO</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H112" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I112" t="str">
         <v>No</v>
@@ -3650,28 +3650,28 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>Shanta Samlal</v>
+        <v>Rohan Bandla</v>
       </c>
       <c r="B113" t="str">
-        <v>shanta.samlal@pwc.com</v>
+        <v/>
       </c>
       <c r="C113" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D113" t="str">
-        <v>PMO</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E113" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F113" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G113" t="str">
-        <v>PMO</v>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H113" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I113" t="str">
         <v>No</v>
@@ -3679,28 +3679,28 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>Aakanksha</v>
+        <v>Russell Stein</v>
       </c>
       <c r="B114" t="str">
-        <v/>
+        <v>russell.stein@pwc.com</v>
       </c>
       <c r="C114" t="str">
-        <v>Infosys</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D114" t="str">
-        <v>QA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E114" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F114" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="G114" t="str">
-        <v>Outage</v>
+        <v>Billing &amp; Usage</v>
       </c>
       <c r="H114" t="str">
-        <v>Dev POD 5/Pornima</v>
+        <v>Dev POD 1/Shreya</v>
       </c>
       <c r="I114" t="str">
         <v>No</v>
@@ -3708,28 +3708,28 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>Argene Francisco</v>
+        <v>Sahithi Manne</v>
       </c>
       <c r="B115" t="str">
         <v/>
       </c>
       <c r="C115" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D115" t="str">
-        <v>QA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E115" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F115" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G115" t="str">
-        <v>Move In, Transfer</v>
+        <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
       </c>
       <c r="H115" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I115" t="str">
         <v>No</v>
@@ -3737,25 +3737,25 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>Argene M. Francisco</v>
+        <v>Courtney Hawkins</v>
       </c>
       <c r="B116" t="str">
-        <v>argene.francisco@pwc.com</v>
+        <v>courtney.c.hawkins@pwc.com</v>
       </c>
       <c r="C116" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D116" t="str">
-        <v>QA</v>
+        <v>PMO</v>
       </c>
       <c r="E116" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F116" t="str">
         <v>All</v>
       </c>
       <c r="G116" t="str">
-        <v>Move In/Transfer</v>
+        <v>PMO</v>
       </c>
       <c r="H116" t="str">
         <v/>
@@ -3766,28 +3766,28 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>Ashit Prashant Golwala</v>
+        <v>Paarth Sonwaney</v>
       </c>
       <c r="B117" t="str">
-        <v>ashit.prashant.golwala@pwc.com</v>
+        <v>paarth.sonwaney@pwc.com</v>
       </c>
       <c r="C117" t="str">
-        <v>Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D117" t="str">
-        <v>QA</v>
+        <v>PMO</v>
       </c>
       <c r="E117" t="str">
-        <v>IR4</v>
+        <v>Leadership</v>
       </c>
       <c r="F117" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G117" t="str">
-        <v>Energy Management</v>
+        <v>PMO</v>
       </c>
       <c r="H117" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I117" t="str">
         <v>No</v>
@@ -3795,25 +3795,25 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Bhyravabhotla Naga Lakshmi Sirisha</v>
+        <v>Shanta Samlal</v>
       </c>
       <c r="B118" t="str">
-        <v>bhyravabhotla.naga.lakshmi.sirisha@pwc.com</v>
+        <v>shanta.samlal@pwc.com</v>
       </c>
       <c r="C118" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D118" t="str">
-        <v>QA</v>
+        <v>PMO</v>
       </c>
       <c r="E118" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F118" t="str">
         <v>All</v>
       </c>
       <c r="G118" t="str">
-        <v>Move In/Move Out</v>
+        <v>PMO</v>
       </c>
       <c r="H118" t="str">
         <v/>
@@ -3824,7 +3824,7 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Diksha</v>
+        <v>Aakanksha</v>
       </c>
       <c r="B119" t="str">
         <v/>
@@ -3853,7 +3853,7 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Dnyanesh Prakash Painjan</v>
+        <v>Argene Francisco</v>
       </c>
       <c r="B120" t="str">
         <v/>
@@ -3882,13 +3882,13 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Dnyanesh Prakash Painjane</v>
+        <v>Argene M. Francisco</v>
       </c>
       <c r="B121" t="str">
-        <v>dnyanesh.prakash.painjane@pwc.com</v>
+        <v>argene.francisco@pwc.com</v>
       </c>
       <c r="C121" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D121" t="str">
         <v>QA</v>
@@ -3911,25 +3911,25 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Girlee Alvarado</v>
+        <v>Ashit Golwala</v>
       </c>
       <c r="B122" t="str">
-        <v/>
+        <v>ashit.prashant.golwala@pwc.com</v>
       </c>
       <c r="C122" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D122" t="str">
         <v>QA</v>
       </c>
       <c r="E122" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F122" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G122" t="str">
-        <v>Move Out, Transfer</v>
+        <v>Energy Management</v>
       </c>
       <c r="H122" t="str">
         <v/>
@@ -3940,28 +3940,28 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>Girlee P. Alvarado</v>
+        <v>Ashit Prashant Golwala</v>
       </c>
       <c r="B123" t="str">
-        <v>girlee.alvarado@pwc.com</v>
+        <v/>
       </c>
       <c r="C123" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D123" t="str">
         <v>QA</v>
       </c>
       <c r="E123" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F123" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G123" t="str">
-        <v>Move Out/Transfer</v>
+        <v/>
       </c>
       <c r="H123" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I123" t="str">
         <v>No</v>
@@ -3969,25 +3969,25 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>Grace Nazareno</v>
+        <v>Bhyravabhotla Naga Lakshmi Sirisha</v>
       </c>
       <c r="B124" t="str">
-        <v/>
+        <v>bhyravabhotla.naga.lakshmi.sirisha@pwc.com</v>
       </c>
       <c r="C124" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D124" t="str">
         <v>QA</v>
       </c>
       <c r="E124" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F124" t="str">
         <v>All</v>
       </c>
       <c r="G124" t="str">
-        <v>Payment &amp; Payment Options, Billing Programs</v>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H124" t="str">
         <v/>
@@ -3998,28 +3998,28 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>ISH Jacinto</v>
+        <v>Diksha</v>
       </c>
       <c r="B125" t="str">
         <v/>
       </c>
       <c r="C125" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D125" t="str">
         <v>QA</v>
       </c>
       <c r="E125" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.X</v>
       </c>
       <c r="F125" t="str">
-        <v>All</v>
+        <v>IR3.X</v>
       </c>
       <c r="G125" t="str">
-        <v>Move Out</v>
+        <v>Outage</v>
       </c>
       <c r="H125" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I125" t="str">
         <v>No</v>
@@ -4027,25 +4027,25 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>Israel L. Jacinto</v>
+        <v>Dnyanesh Prakash Painjan</v>
       </c>
       <c r="B126" t="str">
-        <v>israel.jacinto@pwc.com</v>
+        <v/>
       </c>
       <c r="C126" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D126" t="str">
         <v>QA</v>
       </c>
       <c r="E126" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F126" t="str">
         <v>All</v>
       </c>
       <c r="G126" t="str">
-        <v>Move Out</v>
+        <v>Move In, Transfer</v>
       </c>
       <c r="H126" t="str">
         <v/>
@@ -4056,13 +4056,13 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>Keerthana Manjunath</v>
+        <v>Dnyanesh Prakash Painjane</v>
       </c>
       <c r="B127" t="str">
-        <v/>
+        <v>dnyanesh.prakash.painjane@pwc.com</v>
       </c>
       <c r="C127" t="str">
-        <v>Infosys</v>
+        <v>Associate</v>
       </c>
       <c r="D127" t="str">
         <v>QA</v>
@@ -4074,7 +4074,7 @@
         <v>All</v>
       </c>
       <c r="G127" t="str">
-        <v>Transfer</v>
+        <v>Move In/Transfer</v>
       </c>
       <c r="H127" t="str">
         <v/>
@@ -4085,28 +4085,28 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>Lokesh Sai</v>
+        <v>Girlee Alvarado</v>
       </c>
       <c r="B128" t="str">
-        <v>lokesh.sai@pwc.com</v>
+        <v/>
       </c>
       <c r="C128" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D128" t="str">
         <v>QA</v>
       </c>
       <c r="E128" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F128" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G128" t="str">
-        <v>Energy Management</v>
+        <v>Move Out, Transfer</v>
       </c>
       <c r="H128" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I128" t="str">
         <v>No</v>
@@ -4114,13 +4114,13 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>Maneesha</v>
+        <v>Girlee P. Alvarado</v>
       </c>
       <c r="B129" t="str">
-        <v/>
+        <v>girlee.alvarado@pwc.com</v>
       </c>
       <c r="C129" t="str">
-        <v>Infosys</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D129" t="str">
         <v>QA</v>
@@ -4132,7 +4132,7 @@
         <v>All</v>
       </c>
       <c r="G129" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Move Out/Transfer</v>
       </c>
       <c r="H129" t="str">
         <v/>
@@ -4143,25 +4143,25 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Mary Grace Carinan Nazareno</v>
+        <v>Grace Nazareno</v>
       </c>
       <c r="B130" t="str">
-        <v>mary.grace.nazareno@pwc.com</v>
+        <v/>
       </c>
       <c r="C130" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D130" t="str">
         <v>QA</v>
       </c>
       <c r="E130" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F130" t="str">
         <v>All</v>
       </c>
       <c r="G130" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Payment &amp; Payment Options, Billing Programs</v>
       </c>
       <c r="H130" t="str">
         <v/>
@@ -4172,28 +4172,28 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>Mayand Mani</v>
+        <v>ISH Jacinto</v>
       </c>
       <c r="B131" t="str">
         <v/>
       </c>
       <c r="C131" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D131" t="str">
         <v>QA</v>
       </c>
       <c r="E131" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F131" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G131" t="str">
-        <v>Energy Management</v>
+        <v>Move Out</v>
       </c>
       <c r="H131" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I131" t="str">
         <v>No</v>
@@ -4201,25 +4201,25 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>Mindi Sai Bhavana</v>
+        <v>Israel L. Jacinto</v>
       </c>
       <c r="B132" t="str">
-        <v/>
+        <v>israel.jacinto@pwc.com</v>
       </c>
       <c r="C132" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D132" t="str">
         <v>QA</v>
       </c>
       <c r="E132" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F132" t="str">
         <v>All</v>
       </c>
       <c r="G132" t="str">
-        <v>Case Management</v>
+        <v>Move Out</v>
       </c>
       <c r="H132" t="str">
         <v/>
@@ -4230,13 +4230,13 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>Naga Srilekha Thummalacheruvu</v>
+        <v>Keerthana Manjunath</v>
       </c>
       <c r="B133" t="str">
-        <v>naga.t.thummalacheruvu@pwc.com</v>
+        <v/>
       </c>
       <c r="C133" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D133" t="str">
         <v>QA</v>
@@ -4248,7 +4248,7 @@
         <v>All</v>
       </c>
       <c r="G133" t="str">
-        <v>Move In</v>
+        <v>Transfer</v>
       </c>
       <c r="H133" t="str">
         <v/>
@@ -4259,28 +4259,28 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>Nikita</v>
+        <v>Lokesh Sai</v>
       </c>
       <c r="B134" t="str">
-        <v/>
+        <v>madana.lokesh.dhana.sai@pwc.com</v>
       </c>
       <c r="C134" t="str">
-        <v>Infosys</v>
+        <v>Associate</v>
       </c>
       <c r="D134" t="str">
         <v>QA</v>
       </c>
       <c r="E134" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F134" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G134" t="str">
-        <v>Payment &amp; Payment Options</v>
+        <v>Energy Management</v>
       </c>
       <c r="H134" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I134" t="str">
         <v>No</v>
@@ -4288,7 +4288,7 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Nilesh</v>
+        <v>Maneesha</v>
       </c>
       <c r="B135" t="str">
         <v/>
@@ -4306,7 +4306,7 @@
         <v>All</v>
       </c>
       <c r="G135" t="str">
-        <v>Account Maintenance</v>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H135" t="str">
         <v/>
@@ -4317,25 +4317,25 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>Prasanna</v>
+        <v>Mary Grace Carinan Nazareno</v>
       </c>
       <c r="B136" t="str">
-        <v/>
+        <v>mary.grace.nazareno@pwc.com</v>
       </c>
       <c r="C136" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D136" t="str">
         <v>QA</v>
       </c>
       <c r="E136" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F136" t="str">
         <v>All</v>
       </c>
       <c r="G136" t="str">
-        <v>Billing Programs</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H136" t="str">
         <v/>
@@ -4346,10 +4346,10 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>Prasanna Nangnure</v>
+        <v>Mindi Sai Bhavana</v>
       </c>
       <c r="B137" t="str">
-        <v>prasanna.y.nangnure@pwc.com</v>
+        <v>mindi.sai.bhavana@pwc.com</v>
       </c>
       <c r="C137" t="str">
         <v>Associate</v>
@@ -4358,13 +4358,13 @@
         <v>QA</v>
       </c>
       <c r="E137" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F137" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G137" t="str">
-        <v>Billing Programs</v>
+        <v/>
       </c>
       <c r="H137" t="str">
         <v/>
@@ -4375,13 +4375,13 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>Pratik Mahajan</v>
+        <v>Naga Srilekha Thummalacheruvu</v>
       </c>
       <c r="B138" t="str">
-        <v>pratik.sunil.mahajan@pwc.com</v>
+        <v>naga.t.thummalacheruvu@pwc.com</v>
       </c>
       <c r="C138" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D138" t="str">
         <v>QA</v>
@@ -4393,7 +4393,7 @@
         <v>All</v>
       </c>
       <c r="G138" t="str">
-        <v>Interactions/Search</v>
+        <v>Move In</v>
       </c>
       <c r="H138" t="str">
         <v/>
@@ -4404,25 +4404,25 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>Pritam</v>
+        <v>Navyashree Shantharam</v>
       </c>
       <c r="B139" t="str">
-        <v/>
+        <v>navyashree.s.shantharam@pwc.com</v>
       </c>
       <c r="C139" t="str">
-        <v>Infosys</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D139" t="str">
         <v>QA</v>
       </c>
       <c r="E139" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F139" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G139" t="str">
-        <v>Account Maintenance</v>
+        <v/>
       </c>
       <c r="H139" t="str">
         <v/>
@@ -4433,13 +4433,13 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>Raveendra Reddy</v>
+        <v>Nikita</v>
       </c>
       <c r="B140" t="str">
-        <v>raveendra.t.reddy@pwc.com</v>
+        <v/>
       </c>
       <c r="C140" t="str">
-        <v>Senior Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D140" t="str">
         <v>QA</v>
@@ -4451,7 +4451,7 @@
         <v>All</v>
       </c>
       <c r="G140" t="str">
-        <v>Transfer</v>
+        <v>Payment &amp; Payment Options</v>
       </c>
       <c r="H140" t="str">
         <v/>
@@ -4462,28 +4462,28 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>Sagnik Chakraborty</v>
+        <v>Nilesh</v>
       </c>
       <c r="B141" t="str">
-        <v>sagnik.chakraborty@pwc.com</v>
+        <v/>
       </c>
       <c r="C141" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D141" t="str">
         <v>QA</v>
       </c>
       <c r="E141" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F141" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G141" t="str">
-        <v>Energy Management</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H141" t="str">
-        <v>Dev POD 3/Anurag</v>
+        <v/>
       </c>
       <c r="I141" t="str">
         <v>No</v>
@@ -4491,25 +4491,25 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>Sanjana</v>
+        <v>Prasanna</v>
       </c>
       <c r="B142" t="str">
         <v/>
       </c>
       <c r="C142" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D142" t="str">
         <v>QA</v>
       </c>
       <c r="E142" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F142" t="str">
         <v>All</v>
       </c>
       <c r="G142" t="str">
-        <v>Interactions/Search</v>
+        <v>Billing Programs</v>
       </c>
       <c r="H142" t="str">
         <v/>
@@ -4520,13 +4520,13 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>Smita</v>
+        <v>Prasanna Nangnure</v>
       </c>
       <c r="B143" t="str">
-        <v/>
+        <v>prasanna.y.nangnure@pwc.com</v>
       </c>
       <c r="C143" t="str">
-        <v>Infosys</v>
+        <v>Associate</v>
       </c>
       <c r="D143" t="str">
         <v>QA</v>
@@ -4538,7 +4538,7 @@
         <v>All</v>
       </c>
       <c r="G143" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Billing Programs</v>
       </c>
       <c r="H143" t="str">
         <v/>
@@ -4549,10 +4549,10 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>Sonal Yadav</v>
+        <v>Pratik Mahajan</v>
       </c>
       <c r="B144" t="str">
-        <v>sonal.y.yadav@pwc.com</v>
+        <v>pratik.sunil.mahajan@pwc.com</v>
       </c>
       <c r="C144" t="str">
         <v>Senior Associate</v>
@@ -4567,7 +4567,7 @@
         <v>All</v>
       </c>
       <c r="G144" t="str">
-        <v>Move In/Move Out</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H144" t="str">
         <v/>
@@ -4578,7 +4578,7 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>Venugopal Sinde</v>
+        <v>Pritam</v>
       </c>
       <c r="B145" t="str">
         <v/>
@@ -4596,7 +4596,7 @@
         <v>All</v>
       </c>
       <c r="G145" t="str">
-        <v>Move In/Move Out</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H145" t="str">
         <v/>
@@ -4607,25 +4607,25 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>Vidyashree</v>
+        <v>Raveendra Reddy</v>
       </c>
       <c r="B146" t="str">
-        <v/>
+        <v>raveendra.t.reddy@pwc.com</v>
       </c>
       <c r="C146" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D146" t="str">
         <v>QA</v>
       </c>
       <c r="E146" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F146" t="str">
         <v>All</v>
       </c>
       <c r="G146" t="str">
-        <v>Payment &amp; Payment Options</v>
+        <v>Transfer</v>
       </c>
       <c r="H146" t="str">
         <v/>
@@ -4636,28 +4636,28 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>Vidyashree S R</v>
+        <v>Sagnik Chakraborty</v>
       </c>
       <c r="B147" t="str">
-        <v>vidyashree.s.r@pwc.com</v>
+        <v>sagnik.c.chakraborty@pwc.com</v>
       </c>
       <c r="C147" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D147" t="str">
         <v>QA</v>
       </c>
       <c r="E147" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F147" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G147" t="str">
-        <v>Payment &amp; Payment Options</v>
+        <v>Energy Management</v>
       </c>
       <c r="H147" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I147" t="str">
         <v>No</v>
@@ -4665,16 +4665,16 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>Rajaraman A</v>
+        <v>Sanjana</v>
       </c>
       <c r="B148" t="str">
-        <v>rajaraman.a@pwc.com</v>
+        <v/>
       </c>
       <c r="C148" t="str">
-        <v>Manager</v>
+        <v>Infosys</v>
       </c>
       <c r="D148" t="str">
-        <v>QA Lead</v>
+        <v>QA</v>
       </c>
       <c r="E148" t="str">
         <v>IR3.2</v>
@@ -4683,7 +4683,7 @@
         <v>All</v>
       </c>
       <c r="G148" t="str">
-        <v>QA - All Value Streams</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H148" t="str">
         <v/>
@@ -4694,25 +4694,25 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Tyaga Pati</v>
+        <v>Shreya Maji</v>
       </c>
       <c r="B149" t="str">
-        <v>tyaga.pati@pwc.com</v>
+        <v>shreya.maji@pwc.com</v>
       </c>
       <c r="C149" t="str">
-        <v>Senior Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D149" t="str">
-        <v>Solution Architect</v>
+        <v>QA</v>
       </c>
       <c r="E149" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F149" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G149" t="str">
-        <v>Architecture</v>
+        <v/>
       </c>
       <c r="H149" t="str">
         <v/>
@@ -4723,25 +4723,25 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>Rodolfo Duarte</v>
+        <v>Smita</v>
       </c>
       <c r="B150" t="str">
         <v/>
       </c>
       <c r="C150" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D150" t="str">
-        <v>Team</v>
+        <v>QA</v>
       </c>
       <c r="E150" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F150" t="str">
         <v>All</v>
       </c>
       <c r="G150" t="str">
-        <v/>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H150" t="str">
         <v/>
@@ -4752,25 +4752,25 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>Hemant Jain</v>
+        <v>Sonal Yadav</v>
       </c>
       <c r="B151" t="str">
-        <v>hemant.jain@pwc.com</v>
+        <v>sonal.y.yadav@pwc.com</v>
       </c>
       <c r="C151" t="str">
-        <v>Senior Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D151" t="str">
-        <v>Technical Architect</v>
+        <v>QA</v>
       </c>
       <c r="E151" t="str">
-        <v>Leadership</v>
+        <v>IR3.2</v>
       </c>
       <c r="F151" t="str">
         <v>All</v>
       </c>
       <c r="G151" t="str">
-        <v>Architecture</v>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H151" t="str">
         <v/>
@@ -4781,25 +4781,25 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>Harish Govindareddy</v>
+        <v>Venugopal Sinde</v>
       </c>
       <c r="B152" t="str">
-        <v>harish.govindareddy@pwc.com</v>
+        <v/>
       </c>
       <c r="C152" t="str">
-        <v>Senior Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D152" t="str">
-        <v>Windsurf/Performance Dev</v>
+        <v>QA</v>
       </c>
       <c r="E152" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F152" t="str">
         <v>All</v>
       </c>
       <c r="G152" t="str">
-        <v>Windsurf/Performance</v>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H152" t="str">
         <v/>
@@ -4810,16 +4810,16 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>Sanket Mundargi</v>
+        <v>Vidyashree</v>
       </c>
       <c r="B153" t="str">
-        <v>sanket.mundargi@pwc.com</v>
+        <v/>
       </c>
       <c r="C153" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D153" t="str">
-        <v>Windsurf/Performance Dev</v>
+        <v>QA</v>
       </c>
       <c r="E153" t="str">
         <v>Cross-Functional</v>
@@ -4828,18 +4828,192 @@
         <v>All</v>
       </c>
       <c r="G153" t="str">
+        <v>Payment &amp; Payment Options</v>
+      </c>
+      <c r="H153" t="str">
+        <v/>
+      </c>
+      <c r="I153" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>Vidyashree S R</v>
+      </c>
+      <c r="B154" t="str">
+        <v>vidyashree.s.r@pwc.com</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Senior Associate</v>
+      </c>
+      <c r="D154" t="str">
+        <v>QA</v>
+      </c>
+      <c r="E154" t="str">
+        <v>IR3.2</v>
+      </c>
+      <c r="F154" t="str">
+        <v>All</v>
+      </c>
+      <c r="G154" t="str">
+        <v>Payment &amp; Payment Options</v>
+      </c>
+      <c r="H154" t="str">
+        <v/>
+      </c>
+      <c r="I154" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>Rajaraman A</v>
+      </c>
+      <c r="B155" t="str">
+        <v>rajaraman.a@pwc.com</v>
+      </c>
+      <c r="C155" t="str">
+        <v>Manager</v>
+      </c>
+      <c r="D155" t="str">
+        <v>QA Lead</v>
+      </c>
+      <c r="E155" t="str">
+        <v>IR3.2</v>
+      </c>
+      <c r="F155" t="str">
+        <v>All</v>
+      </c>
+      <c r="G155" t="str">
+        <v>QA - All Value Streams</v>
+      </c>
+      <c r="H155" t="str">
+        <v/>
+      </c>
+      <c r="I155" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>Tyaga Pati</v>
+      </c>
+      <c r="B156" t="str">
+        <v>tyaga.pati@pwc.com</v>
+      </c>
+      <c r="C156" t="str">
+        <v>Senior Manager</v>
+      </c>
+      <c r="D156" t="str">
+        <v>Solution Architect</v>
+      </c>
+      <c r="E156" t="str">
+        <v>Leadership</v>
+      </c>
+      <c r="F156" t="str">
+        <v>All</v>
+      </c>
+      <c r="G156" t="str">
+        <v>Architecture</v>
+      </c>
+      <c r="H156" t="str">
+        <v/>
+      </c>
+      <c r="I156" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>Hemant Jain</v>
+      </c>
+      <c r="B157" t="str">
+        <v>hemant.jain@pwc.com</v>
+      </c>
+      <c r="C157" t="str">
+        <v>Senior Manager</v>
+      </c>
+      <c r="D157" t="str">
+        <v>Technical Architect</v>
+      </c>
+      <c r="E157" t="str">
+        <v>Leadership</v>
+      </c>
+      <c r="F157" t="str">
+        <v>All</v>
+      </c>
+      <c r="G157" t="str">
+        <v>Architecture</v>
+      </c>
+      <c r="H157" t="str">
+        <v/>
+      </c>
+      <c r="I157" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>Harish Govindareddy</v>
+      </c>
+      <c r="B158" t="str">
+        <v>harish.govindareddy@pwc.com</v>
+      </c>
+      <c r="C158" t="str">
+        <v>Senior Associate</v>
+      </c>
+      <c r="D158" t="str">
+        <v>Windsurf/Performance Dev</v>
+      </c>
+      <c r="E158" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="F158" t="str">
+        <v>All</v>
+      </c>
+      <c r="G158" t="str">
         <v>Windsurf/Performance</v>
       </c>
-      <c r="H153" t="str">
-        <v/>
-      </c>
-      <c r="I153" t="str">
+      <c r="H158" t="str">
+        <v/>
+      </c>
+      <c r="I158" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>Sanket Mundargi</v>
+      </c>
+      <c r="B159" t="str">
+        <v>sanket.mundargi@pwc.com</v>
+      </c>
+      <c r="C159" t="str">
+        <v>Associate</v>
+      </c>
+      <c r="D159" t="str">
+        <v>Windsurf/Performance Dev</v>
+      </c>
+      <c r="E159" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="F159" t="str">
+        <v>All</v>
+      </c>
+      <c r="G159" t="str">
+        <v>Windsurf/Performance</v>
+      </c>
+      <c r="H159" t="str">
+        <v/>
+      </c>
+      <c r="I159" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I153"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I159"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add "Planned End Date" column and update JSON data
#VERCEL_SKIP
</commit_message>
<xml_diff>
--- a/public/FPL Staffing.xlsx
+++ b/public/FPL Staffing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pwc-my.sharepoint.com/personal/mayur_murlidhar_kinhekar_pwc_com/Documents/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{097D50CA-A97F-49B7-B19A-63642E9A61BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{116313E0-0013-4020-B2E2-2667E9991886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1289" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="379">
   <si>
     <t>Name</t>
   </si>
@@ -1138,6 +1138,42 @@
   </si>
   <si>
     <t>mayand.mani@pwc.com</t>
+  </si>
+  <si>
+    <t>08/24/2026</t>
+  </si>
+  <si>
+    <t>08/31/2026</t>
+  </si>
+  <si>
+    <t>07/27/2026</t>
+  </si>
+  <si>
+    <t>07/20/2026</t>
+  </si>
+  <si>
+    <t>06/15/2026</t>
+  </si>
+  <si>
+    <t>10/26/2026</t>
+  </si>
+  <si>
+    <t>08/03/2026</t>
+  </si>
+  <si>
+    <t>06/29/2026</t>
+  </si>
+  <si>
+    <t>08/10/2026</t>
+  </si>
+  <si>
+    <t>06/01/2026</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>11/23/2026</t>
   </si>
 </sst>
 </file>
@@ -1704,7 +1740,9 @@
       <c r="G2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -1728,7 +1766,9 @@
       <c r="G3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -1752,7 +1792,9 @@
       <c r="G4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
@@ -1776,7 +1818,9 @@
       <c r="G5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>368</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
@@ -1800,7 +1844,9 @@
       <c r="G6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
@@ -1824,7 +1870,9 @@
       <c r="G7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>369</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
@@ -1848,7 +1896,9 @@
       <c r="G8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>370</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
@@ -1872,7 +1922,9 @@
       <c r="G9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="2"/>
+      <c r="H9" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
@@ -1896,7 +1948,9 @@
       <c r="G10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
@@ -1920,7 +1974,9 @@
       <c r="G11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H11" s="2"/>
+      <c r="H11" s="2" t="s">
+        <v>368</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
@@ -1944,7 +2000,9 @@
       <c r="G12" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
@@ -1968,7 +2026,9 @@
       <c r="G13" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H13" s="6"/>
+      <c r="H13" s="6" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
@@ -1992,7 +2052,9 @@
       <c r="G14" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H14" s="2"/>
+      <c r="H14" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
@@ -2016,7 +2078,9 @@
       <c r="G15" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H15" s="2"/>
+      <c r="H15" s="2" t="s">
+        <v>372</v>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
@@ -2040,7 +2104,9 @@
       <c r="G16" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H16" s="2"/>
+      <c r="H16" s="2" t="s">
+        <v>373</v>
+      </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
@@ -2064,7 +2130,9 @@
       <c r="G17" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H17" s="2"/>
+      <c r="H17" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
@@ -2088,7 +2156,9 @@
       <c r="G18" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
@@ -2112,7 +2182,9 @@
       <c r="G19" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H19" s="2"/>
+      <c r="H19" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
@@ -2136,7 +2208,9 @@
       <c r="G20" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H20" s="2"/>
+      <c r="H20" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
@@ -2160,7 +2234,9 @@
       <c r="G21" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H21" s="2"/>
+      <c r="H21" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
@@ -2184,7 +2260,9 @@
       <c r="G22" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H22" s="6"/>
+      <c r="H22" s="6" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
@@ -2208,7 +2286,9 @@
       <c r="G23" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="H23" s="2"/>
+      <c r="H23" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
@@ -2232,7 +2312,9 @@
       <c r="G24" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="H24" s="2"/>
+      <c r="H24" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
@@ -2256,7 +2338,9 @@
       <c r="G25" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="H25" s="2"/>
+      <c r="H25" s="2" t="s">
+        <v>370</v>
+      </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
@@ -2280,7 +2364,9 @@
       <c r="G26" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="H26" s="2"/>
+      <c r="H26" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
@@ -2304,7 +2390,9 @@
       <c r="G27" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="2"/>
+      <c r="H27" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
@@ -2352,7 +2440,9 @@
       <c r="G29" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="H29" s="2"/>
+      <c r="H29" s="2" t="s">
+        <v>370</v>
+      </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
@@ -2376,7 +2466,9 @@
       <c r="G30" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H30" s="2"/>
+      <c r="H30" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
@@ -2400,7 +2492,9 @@
       <c r="G31" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H31" s="2"/>
+      <c r="H31" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
@@ -2448,7 +2542,9 @@
       <c r="G33" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="H33" s="2"/>
+      <c r="H33" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
@@ -2472,7 +2568,9 @@
       <c r="G34" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="H34" s="2"/>
+      <c r="H34" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
@@ -2496,7 +2594,9 @@
       <c r="G35" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="H35" s="2"/>
+      <c r="H35" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
@@ -2520,7 +2620,9 @@
       <c r="G36" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="H36" s="2"/>
+      <c r="H36" s="2" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
@@ -2544,7 +2646,9 @@
       <c r="G37" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="H37" s="2"/>
+      <c r="H37" s="2" t="s">
+        <v>375</v>
+      </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="4" t="s">
@@ -2592,7 +2696,9 @@
       <c r="G39" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="H39" s="2"/>
+      <c r="H39" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
@@ -2638,7 +2744,9 @@
       <c r="G41" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="H41" s="2"/>
+      <c r="H41" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="4" t="s">
@@ -2662,7 +2770,9 @@
       <c r="G42" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="H42" s="2"/>
+      <c r="H42" s="2" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="s">
@@ -2686,7 +2796,9 @@
       <c r="G43" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="H43" s="2"/>
+      <c r="H43" s="2" t="s">
+        <v>376</v>
+      </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
@@ -2732,7 +2844,9 @@
       <c r="G45" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="H45" s="2"/>
+      <c r="H45" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
@@ -2756,7 +2870,9 @@
       <c r="G46" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="H46" s="2"/>
+      <c r="H46" s="2" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
@@ -2780,7 +2896,9 @@
       <c r="G47" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="H47" s="2"/>
+      <c r="H47" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
@@ -2826,7 +2944,9 @@
       <c r="G49" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="H49" s="2"/>
+      <c r="H49" s="2" t="s">
+        <v>371</v>
+      </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
@@ -2850,7 +2970,9 @@
       <c r="G50" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="H50" s="2"/>
+      <c r="H50" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
@@ -2896,7 +3018,9 @@
       <c r="G52" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="H52" s="2"/>
+      <c r="H52" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="4" t="s">
@@ -2986,7 +3110,9 @@
       <c r="G56" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="H56" s="2"/>
+      <c r="H56" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="4" t="s">
@@ -3010,7 +3136,9 @@
       <c r="G57" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="H57" s="2"/>
+      <c r="H57" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="4" t="s">
@@ -3056,7 +3184,9 @@
       <c r="G59" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="H59" s="2"/>
+      <c r="H59" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
@@ -3080,7 +3210,9 @@
       <c r="G60" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="H60" s="2"/>
+      <c r="H60" s="2" t="s">
+        <v>370</v>
+      </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
@@ -3102,7 +3234,9 @@
       <c r="G61" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="H61" s="2"/>
+      <c r="H61" s="2" t="s">
+        <v>375</v>
+      </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
@@ -3126,7 +3260,9 @@
       <c r="G62" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="H62" s="2"/>
+      <c r="H62" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
@@ -3150,7 +3286,9 @@
       <c r="G63" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="H63" s="2"/>
+      <c r="H63" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
@@ -3216,7 +3354,9 @@
       <c r="G66" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="H66" s="2"/>
+      <c r="H66" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
@@ -3240,7 +3380,9 @@
       <c r="G67" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="H67" s="2"/>
+      <c r="H67" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
@@ -3264,7 +3406,9 @@
       <c r="G68" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="H68" s="2"/>
+      <c r="H68" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
@@ -3288,7 +3432,9 @@
       <c r="G69" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="H69" s="2"/>
+      <c r="H69" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
@@ -3310,7 +3456,9 @@
       <c r="G70" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H70" s="2"/>
+      <c r="H70" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
@@ -3334,7 +3482,9 @@
       <c r="G71" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H71" s="2"/>
+      <c r="H71" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
@@ -3358,7 +3508,9 @@
       <c r="G72" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H72" s="2"/>
+      <c r="H72" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
@@ -3382,7 +3534,9 @@
       <c r="G73" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H73" s="2"/>
+      <c r="H73" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
@@ -3406,7 +3560,9 @@
       <c r="G74" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="H74" s="2"/>
+      <c r="H74" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
@@ -3430,7 +3586,9 @@
       <c r="G75" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="H75" s="2"/>
+      <c r="H75" s="2" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
@@ -3454,7 +3612,9 @@
       <c r="G76" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="H76" s="3"/>
+      <c r="H76" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
@@ -3502,7 +3662,9 @@
       <c r="G78" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="H78" s="3"/>
+      <c r="H78" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
@@ -3526,7 +3688,9 @@
       <c r="G79" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="H79" s="3"/>
+      <c r="H79" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
@@ -3550,7 +3714,9 @@
       <c r="G80" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="H80" s="3"/>
+      <c r="H80" s="3" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
@@ -3574,7 +3740,9 @@
       <c r="G81" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="H81" s="3"/>
+      <c r="H81" s="3" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
@@ -3598,7 +3766,9 @@
       <c r="G82" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="H82" s="3"/>
+      <c r="H82" s="3" t="s">
+        <v>370</v>
+      </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
@@ -3622,7 +3792,9 @@
       <c r="G83" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="H83" s="3"/>
+      <c r="H83" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
@@ -3646,7 +3818,9 @@
       <c r="G84" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="H84" s="3"/>
+      <c r="H84" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
@@ -3670,7 +3844,9 @@
       <c r="G85" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="H85" s="3"/>
+      <c r="H85" s="3" t="s">
+        <v>372</v>
+      </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
@@ -3694,7 +3870,9 @@
       <c r="G86" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="H86" s="3"/>
+      <c r="H86" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
@@ -3718,7 +3896,9 @@
       <c r="G87" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="H87" s="3"/>
+      <c r="H87" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
@@ -3742,7 +3922,9 @@
       <c r="G88" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="H88" s="3"/>
+      <c r="H88" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
@@ -3766,7 +3948,9 @@
       <c r="G89" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="H89" s="3"/>
+      <c r="H89" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
@@ -3790,7 +3974,9 @@
       <c r="G90" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="H90" s="3"/>
+      <c r="H90" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
@@ -3814,7 +4000,9 @@
       <c r="G91" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="H91" s="3"/>
+      <c r="H91" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
@@ -3838,7 +4026,9 @@
       <c r="G92" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="H92" s="3"/>
+      <c r="H92" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
@@ -3862,7 +4052,9 @@
       <c r="G93" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="H93" s="3"/>
+      <c r="H93" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
@@ -3886,7 +4078,9 @@
       <c r="G94" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="H94" s="3"/>
+      <c r="H94" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
@@ -3910,7 +4104,9 @@
       <c r="G95" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="H95" s="3"/>
+      <c r="H95" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
@@ -3934,7 +4130,9 @@
       <c r="G96" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="H96" s="3"/>
+      <c r="H96" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
@@ -3958,7 +4156,9 @@
       <c r="G97" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="H97" s="3"/>
+      <c r="H97" s="3" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
@@ -4030,7 +4230,9 @@
       <c r="G100" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="H100" s="3"/>
+      <c r="H100" s="3" t="s">
+        <v>376</v>
+      </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
@@ -4052,7 +4254,9 @@
         <v>179</v>
       </c>
       <c r="G101" s="3"/>
-      <c r="H101" s="3"/>
+      <c r="H101" s="3" t="s">
+        <v>369</v>
+      </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
@@ -4074,7 +4278,9 @@
         <v>179</v>
       </c>
       <c r="G102" s="3"/>
-      <c r="H102" s="3"/>
+      <c r="H102" s="3" t="s">
+        <v>376</v>
+      </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
@@ -4098,7 +4304,9 @@
       <c r="G103" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="H103" s="3"/>
+      <c r="H103" s="3" t="s">
+        <v>376</v>
+      </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
@@ -4144,7 +4352,9 @@
         <v>179</v>
       </c>
       <c r="G105" s="3"/>
-      <c r="H105" s="3"/>
+      <c r="H105" s="3" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
@@ -4168,7 +4378,9 @@
       <c r="G106" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H106" s="3"/>
+      <c r="H106" s="3" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
@@ -4192,7 +4404,9 @@
       <c r="G107" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H107" s="3"/>
+      <c r="H107" s="3" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
@@ -4216,7 +4430,9 @@
       <c r="G108" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="H108" s="5"/>
+      <c r="H108" s="5" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
@@ -4238,7 +4454,9 @@
         <v>179</v>
       </c>
       <c r="G109" s="3"/>
-      <c r="H109" s="3"/>
+      <c r="H109" s="3" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
@@ -4260,7 +4478,9 @@
         <v>179</v>
       </c>
       <c r="G110" s="3"/>
-      <c r="H110" s="3"/>
+      <c r="H110" s="3" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
@@ -4282,7 +4502,9 @@
         <v>179</v>
       </c>
       <c r="G111" s="3"/>
-      <c r="H111" s="3"/>
+      <c r="H111" s="3" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
@@ -4304,7 +4526,9 @@
         <v>179</v>
       </c>
       <c r="G112" s="3"/>
-      <c r="H112" s="3"/>
+      <c r="H112" s="3" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
@@ -4326,7 +4550,9 @@
         <v>179</v>
       </c>
       <c r="G113" s="3"/>
-      <c r="H113" s="3"/>
+      <c r="H113" s="3" t="s">
+        <v>377</v>
+      </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
@@ -4350,7 +4576,9 @@
       <c r="G114" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="H114" s="5"/>
+      <c r="H114" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
@@ -4374,7 +4602,9 @@
       <c r="G115" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="H115" s="5"/>
+      <c r="H115" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
@@ -4398,7 +4628,9 @@
       <c r="G116" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="H116" s="5"/>
+      <c r="H116" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
@@ -4422,7 +4654,9 @@
       <c r="G117" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="H117" s="5"/>
+      <c r="H117" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
@@ -4446,7 +4680,9 @@
       <c r="G118" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="H118" s="5"/>
+      <c r="H118" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
@@ -4470,7 +4706,9 @@
       <c r="G119" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="H119" s="5"/>
+      <c r="H119" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
@@ -4492,7 +4730,9 @@
         <v>179</v>
       </c>
       <c r="G120" s="5"/>
-      <c r="H120" s="5"/>
+      <c r="H120" t="s">
+        <v>378</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>